<commit_message>
chore: cập nhật file sao kê theo tháng, bỏ file khoá tạm của Excel
File ~$sao-ke-co-dinh-theo-thang-va-tai-khoan.xlsx là file khoá Excel tạo ra
lúc đang mở, lần trước bị `git add -A` quét vào kho. Excel đóng thì nó tự
mất, nên gỡ luôn khỏi kho.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/sao-ke-co-dinh-theo-thang-va-tai-khoan.xlsx
+++ b/data/sao-ke-co-dinh-theo-thang-va-tai-khoan.xlsx
@@ -1,13 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10914"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D03A6C8-BD96-4346-A81F-FF01D7ED9D12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="780" windowWidth="41120" windowHeight="24600" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Theo tháng và tài khoản" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Chi tiết từng dòng" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Phần mềm ngoài sao kê" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="Ghi chú" state="visible" r:id="rId7"/>
+    <sheet name="Theo tháng và tài khoản" sheetId="1" r:id="rId1"/>
+    <sheet name="Chi tiết từng dòng" sheetId="2" r:id="rId2"/>
+    <sheet name="Phần mềm ngoài sao kê" sheetId="3" r:id="rId3"/>
+    <sheet name="Ghi chú" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -175,21 +179,34 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="ＭＳ Ｐゴシック"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="ＭＳ Ｐゴシック"/>
+      <charset val="128"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <name val="ＭＳ Ｐゴシック"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <sz val="6"/>
+      <name val="ＭＳ Ｐゴシック"/>
+      <family val="3"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="8">
@@ -242,7 +259,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -265,9 +282,45 @@
     <xf numFmtId="3" fontId="2" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="標準" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -603,40 +656,40 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M16"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="13" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" s="1" customFormat="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2" t="s">
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2" t="s">
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2" t="s">
+      <c r="I1" s="18"/>
+      <c r="J1" s="18"/>
+      <c r="K1" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="L1" s="2"/>
-      <c r="M1" s="2"/>
-    </row>
-    <row r="2" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="L1" s="18"/>
+      <c r="M1" s="18"/>
+    </row>
+    <row r="2" spans="1:13" s="3" customFormat="1">
       <c r="A2" s="4" t="s">
         <v>5</v>
       </c>
@@ -677,7 +730,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13">
       <c r="A3" s="5" t="s">
         <v>9</v>
       </c>
@@ -718,7 +771,7 @@
         <v>2500</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13">
       <c r="A4" s="5" t="s">
         <v>10</v>
       </c>
@@ -759,7 +812,7 @@
         <v>21900</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13">
       <c r="A5" s="7" t="s">
         <v>11</v>
       </c>
@@ -800,7 +853,7 @@
         <v>101948</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13">
       <c r="A6" s="5" t="s">
         <v>12</v>
       </c>
@@ -841,7 +894,7 @@
         <v>36250</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13">
       <c r="A7" s="7" t="s">
         <v>13</v>
       </c>
@@ -882,7 +935,7 @@
         <v>52000</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13">
       <c r="A8" s="9" t="s">
         <v>14</v>
       </c>
@@ -923,7 +976,7 @@
         <v>237871</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13">
       <c r="A9" s="9" t="s">
         <v>15</v>
       </c>
@@ -964,7 +1017,7 @@
         <v>262032</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13">
       <c r="A10" s="9" t="s">
         <v>16</v>
       </c>
@@ -1005,7 +1058,7 @@
         <v>268367</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13">
       <c r="A11" s="9" t="s">
         <v>17</v>
       </c>
@@ -1046,7 +1099,7 @@
         <v>288868</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13">
       <c r="A12" s="9" t="s">
         <v>18</v>
       </c>
@@ -1087,7 +1140,7 @@
         <v>340938</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13">
       <c r="A13" s="9" t="s">
         <v>19</v>
       </c>
@@ -1128,7 +1181,7 @@
         <v>430438</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13">
       <c r="A14" s="5" t="s">
         <v>20</v>
       </c>
@@ -1169,7 +1222,7 @@
         <v>32902</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13">
       <c r="A15" s="11" t="s">
         <v>21</v>
       </c>
@@ -1210,7 +1263,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:13" s="13" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" s="13" customFormat="1">
       <c r="A16" s="14" t="s">
         <v>22</v>
       </c>
@@ -1258,1089 +1311,1092 @@
     <mergeCell ref="H1:J1"/>
     <mergeCell ref="K1:M1"/>
   </mergeCells>
+  <phoneticPr fontId="3"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:K30"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="23" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="13" customWidth="1"/>
-    <col min="4" max="5" width="20" style="16" customWidth="1"/>
-    <col min="6" max="6" width="15" style="16" customWidth="1"/>
-    <col min="7" max="7" width="17" customWidth="1"/>
-    <col min="8" max="8" width="21" style="16" customWidth="1"/>
-    <col min="9" max="9" width="18" style="16" customWidth="1"/>
-    <col min="10" max="10" width="18" customWidth="1"/>
-    <col min="11" max="11" width="14" style="16" customWidth="1"/>
+    <col min="1" max="1" width="10" style="24" customWidth="1"/>
+    <col min="2" max="2" width="16" style="24" customWidth="1"/>
+    <col min="3" max="3" width="13" style="24" customWidth="1"/>
+    <col min="4" max="5" width="20" style="29" customWidth="1"/>
+    <col min="6" max="6" width="15" style="29" customWidth="1"/>
+    <col min="7" max="7" width="17" style="24" customWidth="1"/>
+    <col min="8" max="8" width="21" style="29" customWidth="1"/>
+    <col min="9" max="9" width="18" style="29" customWidth="1"/>
+    <col min="10" max="10" width="18" style="24" customWidth="1"/>
+    <col min="11" max="11" width="14" style="29" customWidth="1"/>
+    <col min="12" max="16384" width="8.83203125" style="24"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:11" s="21" customFormat="1" ht="23" customHeight="1">
+      <c r="A1" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="E1" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="F1" s="17" t="s">
+      <c r="F1" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="H1" s="17" t="s">
+      <c r="H1" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="I1" s="17" t="s">
+      <c r="I1" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="K1" s="17" t="s">
+      <c r="K1" s="20" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+    <row r="2" spans="1:11" ht="23" customHeight="1">
+      <c r="A2" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="5">
+      <c r="C2" s="22">
         <v>1</v>
       </c>
-      <c r="D2" s="6">
+      <c r="D2" s="23">
         <v>2500</v>
       </c>
-      <c r="E2" s="6">
-        <v>0</v>
-      </c>
-      <c r="F2" s="6">
+      <c r="E2" s="23">
+        <v>0</v>
+      </c>
+      <c r="F2" s="23">
         <v>2500</v>
       </c>
-      <c r="G2" s="5">
-        <v>0</v>
-      </c>
-      <c r="H2" s="6">
-        <v>0</v>
-      </c>
-      <c r="I2" s="6">
-        <v>0</v>
-      </c>
-      <c r="J2" s="5">
-        <v>0</v>
-      </c>
-      <c r="K2" s="6">
+      <c r="G2" s="22">
+        <v>0</v>
+      </c>
+      <c r="H2" s="23">
+        <v>0</v>
+      </c>
+      <c r="I2" s="23">
+        <v>0</v>
+      </c>
+      <c r="J2" s="22">
+        <v>0</v>
+      </c>
+      <c r="K2" s="23">
         <v>2500</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
+    <row r="3" spans="1:11" ht="23" customHeight="1">
+      <c r="A3" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="5">
+      <c r="C3" s="22">
         <v>1</v>
       </c>
-      <c r="D3" s="6">
+      <c r="D3" s="23">
         <v>500</v>
       </c>
-      <c r="E3" s="6">
-        <v>0</v>
-      </c>
-      <c r="F3" s="6">
+      <c r="E3" s="23">
+        <v>0</v>
+      </c>
+      <c r="F3" s="23">
         <v>500</v>
       </c>
-      <c r="G3" s="5">
-        <v>0</v>
-      </c>
-      <c r="H3" s="6">
-        <v>0</v>
-      </c>
-      <c r="I3" s="6">
-        <v>0</v>
-      </c>
-      <c r="J3" s="5">
-        <v>0</v>
-      </c>
-      <c r="K3" s="6">
+      <c r="G3" s="22">
+        <v>0</v>
+      </c>
+      <c r="H3" s="23">
+        <v>0</v>
+      </c>
+      <c r="I3" s="23">
+        <v>0</v>
+      </c>
+      <c r="J3" s="22">
+        <v>0</v>
+      </c>
+      <c r="K3" s="23">
         <v>500</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
+    <row r="4" spans="1:11" ht="23" customHeight="1">
+      <c r="A4" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="7">
+      <c r="C4" s="25">
         <v>6</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="26">
         <v>21400</v>
       </c>
-      <c r="E4" s="8">
-        <v>0</v>
-      </c>
-      <c r="F4" s="8">
+      <c r="E4" s="26">
+        <v>0</v>
+      </c>
+      <c r="F4" s="26">
         <v>21400</v>
       </c>
-      <c r="G4" s="7">
+      <c r="G4" s="25">
         <v>3</v>
       </c>
-      <c r="H4" s="8">
+      <c r="H4" s="26">
         <v>5500</v>
       </c>
-      <c r="I4" s="8">
-        <v>0</v>
-      </c>
-      <c r="J4" s="7">
-        <v>0</v>
-      </c>
-      <c r="K4" s="8">
+      <c r="I4" s="26">
+        <v>0</v>
+      </c>
+      <c r="J4" s="25">
+        <v>0</v>
+      </c>
+      <c r="K4" s="26">
         <v>21400</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
+    <row r="5" spans="1:11" ht="23" customHeight="1">
+      <c r="A5" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5" s="22">
         <v>1</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="23">
         <v>7700</v>
       </c>
-      <c r="E5" s="6">
-        <v>0</v>
-      </c>
-      <c r="F5" s="6">
+      <c r="E5" s="23">
+        <v>0</v>
+      </c>
+      <c r="F5" s="23">
         <v>7700</v>
       </c>
-      <c r="G5" s="5">
-        <v>0</v>
-      </c>
-      <c r="H5" s="6">
-        <v>0</v>
-      </c>
-      <c r="I5" s="6">
-        <v>0</v>
-      </c>
-      <c r="J5" s="5">
-        <v>0</v>
-      </c>
-      <c r="K5" s="6">
+      <c r="G5" s="22">
+        <v>0</v>
+      </c>
+      <c r="H5" s="23">
+        <v>0</v>
+      </c>
+      <c r="I5" s="23">
+        <v>0</v>
+      </c>
+      <c r="J5" s="22">
+        <v>0</v>
+      </c>
+      <c r="K5" s="23">
         <v>7700</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
+    <row r="6" spans="1:11" ht="23" customHeight="1">
+      <c r="A6" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="7">
+      <c r="C6" s="25">
         <v>26</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="26">
         <v>94248</v>
       </c>
-      <c r="E6" s="8">
-        <v>0</v>
-      </c>
-      <c r="F6" s="8">
+      <c r="E6" s="26">
+        <v>0</v>
+      </c>
+      <c r="F6" s="26">
         <v>94248</v>
       </c>
-      <c r="G6" s="7">
+      <c r="G6" s="25">
         <v>2</v>
       </c>
-      <c r="H6" s="8">
+      <c r="H6" s="26">
         <v>3100</v>
       </c>
-      <c r="I6" s="8">
-        <v>0</v>
-      </c>
-      <c r="J6" s="7">
-        <v>0</v>
-      </c>
-      <c r="K6" s="8">
+      <c r="I6" s="26">
+        <v>0</v>
+      </c>
+      <c r="J6" s="25">
+        <v>0</v>
+      </c>
+      <c r="K6" s="26">
         <v>94248</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
+    <row r="7" spans="1:11" ht="23" customHeight="1">
+      <c r="A7" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="22">
         <v>3</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="23">
         <v>18850</v>
       </c>
-      <c r="E7" s="6">
-        <v>0</v>
-      </c>
-      <c r="F7" s="6">
+      <c r="E7" s="23">
+        <v>0</v>
+      </c>
+      <c r="F7" s="23">
         <v>18850</v>
       </c>
-      <c r="G7" s="5">
+      <c r="G7" s="22">
         <v>3</v>
       </c>
-      <c r="H7" s="6">
+      <c r="H7" s="23">
         <v>18850</v>
       </c>
-      <c r="I7" s="6">
+      <c r="I7" s="23">
         <v>12000</v>
       </c>
-      <c r="J7" s="5">
+      <c r="J7" s="22">
         <v>6</v>
       </c>
-      <c r="K7" s="6">
+      <c r="K7" s="23">
         <v>6850</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
+    <row r="8" spans="1:11" ht="23" customHeight="1">
+      <c r="A8" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="C8" s="7">
+      <c r="C8" s="25">
         <v>43</v>
       </c>
-      <c r="D8" s="8">
+      <c r="D8" s="26">
         <v>143900</v>
       </c>
-      <c r="E8" s="8">
-        <v>0</v>
-      </c>
-      <c r="F8" s="8">
+      <c r="E8" s="26">
+        <v>0</v>
+      </c>
+      <c r="F8" s="26">
         <v>143900</v>
       </c>
-      <c r="G8" s="7">
+      <c r="G8" s="25">
         <v>42</v>
       </c>
-      <c r="H8" s="8">
+      <c r="H8" s="26">
         <v>141900</v>
       </c>
-      <c r="I8" s="8">
+      <c r="I8" s="26">
         <v>114500</v>
       </c>
-      <c r="J8" s="7">
+      <c r="J8" s="25">
         <v>61</v>
       </c>
-      <c r="K8" s="8">
+      <c r="K8" s="26">
         <v>29400</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" s="5" t="s">
+    <row r="9" spans="1:11" ht="23" customHeight="1">
+      <c r="A9" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="C9" s="5">
+      <c r="C9" s="22">
         <v>5</v>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="23">
         <v>18500</v>
       </c>
-      <c r="E9" s="6">
-        <v>0</v>
-      </c>
-      <c r="F9" s="6">
+      <c r="E9" s="23">
+        <v>0</v>
+      </c>
+      <c r="F9" s="23">
         <v>18500</v>
       </c>
-      <c r="G9" s="5">
+      <c r="G9" s="22">
         <v>5</v>
       </c>
-      <c r="H9" s="6">
+      <c r="H9" s="23">
         <v>18500</v>
       </c>
-      <c r="I9" s="6">
+      <c r="I9" s="23">
         <v>16500</v>
       </c>
-      <c r="J9" s="5">
+      <c r="J9" s="22">
         <v>9</v>
       </c>
-      <c r="K9" s="6">
+      <c r="K9" s="23">
         <v>2000</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
+    <row r="10" spans="1:11" ht="23" customHeight="1">
+      <c r="A10" s="25" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="C10" s="7">
+      <c r="C10" s="25">
         <v>44</v>
       </c>
-      <c r="D10" s="8">
+      <c r="D10" s="26">
         <v>158000</v>
       </c>
-      <c r="E10" s="8">
-        <v>0</v>
-      </c>
-      <c r="F10" s="8">
+      <c r="E10" s="26">
+        <v>0</v>
+      </c>
+      <c r="F10" s="26">
         <v>158000</v>
       </c>
-      <c r="G10" s="7">
+      <c r="G10" s="25">
         <v>43</v>
       </c>
-      <c r="H10" s="8">
+      <c r="H10" s="26">
         <v>146850</v>
       </c>
-      <c r="I10" s="8">
+      <c r="I10" s="26">
         <v>108000</v>
       </c>
-      <c r="J10" s="7">
+      <c r="J10" s="25">
         <v>56</v>
       </c>
-      <c r="K10" s="8">
+      <c r="K10" s="26">
         <v>50000</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
+    <row r="11" spans="1:11" ht="23" customHeight="1">
+      <c r="A11" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="C11" s="5">
+      <c r="C11" s="22">
         <v>11</v>
       </c>
-      <c r="D11" s="6">
+      <c r="D11" s="23">
         <v>28000</v>
       </c>
-      <c r="E11" s="6">
-        <v>0</v>
-      </c>
-      <c r="F11" s="6">
+      <c r="E11" s="23">
+        <v>0</v>
+      </c>
+      <c r="F11" s="23">
         <v>28000</v>
       </c>
-      <c r="G11" s="5">
+      <c r="G11" s="22">
         <v>11</v>
       </c>
-      <c r="H11" s="6">
+      <c r="H11" s="23">
         <v>28000</v>
       </c>
-      <c r="I11" s="6">
+      <c r="I11" s="23">
         <v>18000</v>
       </c>
-      <c r="J11" s="5">
+      <c r="J11" s="22">
         <v>9</v>
       </c>
-      <c r="K11" s="6">
+      <c r="K11" s="23">
         <v>10000</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="9" t="s">
+    <row r="12" spans="1:11" ht="23" customHeight="1">
+      <c r="A12" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="C12" s="9">
+      <c r="C12" s="27">
         <v>75</v>
       </c>
-      <c r="D12" s="10">
+      <c r="D12" s="28">
         <v>339471</v>
       </c>
-      <c r="E12" s="10">
-        <v>0</v>
-      </c>
-      <c r="F12" s="10">
+      <c r="E12" s="28">
+        <v>0</v>
+      </c>
+      <c r="F12" s="28">
         <v>339471</v>
       </c>
-      <c r="G12" s="9">
+      <c r="G12" s="27">
         <v>71</v>
       </c>
-      <c r="H12" s="10">
+      <c r="H12" s="28">
         <v>307471</v>
       </c>
-      <c r="I12" s="10">
+      <c r="I12" s="28">
         <v>111600</v>
       </c>
-      <c r="J12" s="9">
+      <c r="J12" s="27">
         <v>61</v>
       </c>
-      <c r="K12" s="10">
+      <c r="K12" s="28">
         <v>227871</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" s="5" t="s">
+    <row r="13" spans="1:11" ht="23" customHeight="1">
+      <c r="A13" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="C13" s="5">
+      <c r="C13" s="22">
         <v>73</v>
       </c>
-      <c r="D13" s="6">
+      <c r="D13" s="23">
         <v>177469</v>
       </c>
-      <c r="E13" s="6">
-        <v>0</v>
-      </c>
-      <c r="F13" s="6">
+      <c r="E13" s="23">
+        <v>0</v>
+      </c>
+      <c r="F13" s="23">
         <v>177469</v>
       </c>
-      <c r="G13" s="5">
+      <c r="G13" s="22">
         <v>67</v>
       </c>
-      <c r="H13" s="6">
+      <c r="H13" s="23">
         <v>156469</v>
       </c>
-      <c r="I13" s="6">
+      <c r="I13" s="23">
         <v>189000</v>
       </c>
-      <c r="J13" s="5">
+      <c r="J13" s="22">
         <v>101</v>
       </c>
-      <c r="K13" s="6">
+      <c r="K13" s="23">
         <v>-11531</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="5" t="s">
+    <row r="14" spans="1:11" ht="23" customHeight="1">
+      <c r="A14" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="C14" s="5">
-        <v>0</v>
-      </c>
-      <c r="D14" s="6">
-        <v>0</v>
-      </c>
-      <c r="E14" s="6">
-        <v>0</v>
-      </c>
-      <c r="F14" s="6">
-        <v>0</v>
-      </c>
-      <c r="G14" s="5">
-        <v>0</v>
-      </c>
-      <c r="H14" s="6">
-        <v>0</v>
-      </c>
-      <c r="I14" s="6">
+      <c r="C14" s="22">
+        <v>0</v>
+      </c>
+      <c r="D14" s="23">
+        <v>0</v>
+      </c>
+      <c r="E14" s="23">
+        <v>0</v>
+      </c>
+      <c r="F14" s="23">
+        <v>0</v>
+      </c>
+      <c r="G14" s="22">
+        <v>0</v>
+      </c>
+      <c r="H14" s="23">
+        <v>0</v>
+      </c>
+      <c r="I14" s="23">
         <v>2000</v>
       </c>
-      <c r="J14" s="5">
+      <c r="J14" s="22">
         <v>1</v>
       </c>
-      <c r="K14" s="6">
+      <c r="K14" s="23">
         <v>-2000</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A15" s="9" t="s">
+    <row r="15" spans="1:11" ht="23" customHeight="1">
+      <c r="A15" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="C15" s="9">
+      <c r="C15" s="27">
         <v>89</v>
       </c>
-      <c r="D15" s="10">
+      <c r="D15" s="28">
         <v>540963</v>
       </c>
-      <c r="E15" s="10">
-        <v>0</v>
-      </c>
-      <c r="F15" s="10">
+      <c r="E15" s="28">
+        <v>0</v>
+      </c>
+      <c r="F15" s="28">
         <v>540963</v>
       </c>
-      <c r="G15" s="9">
+      <c r="G15" s="27">
         <v>87</v>
       </c>
-      <c r="H15" s="10">
+      <c r="H15" s="28">
         <v>532963</v>
       </c>
-      <c r="I15" s="10">
+      <c r="I15" s="28">
         <v>265400</v>
       </c>
-      <c r="J15" s="9">
+      <c r="J15" s="27">
         <v>138</v>
       </c>
-      <c r="K15" s="10">
+      <c r="K15" s="28">
         <v>275563</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A16" s="7" t="s">
+    <row r="16" spans="1:11" ht="23" customHeight="1">
+      <c r="A16" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="C16" s="7">
+      <c r="C16" s="25">
         <v>126</v>
       </c>
-      <c r="D16" s="8">
+      <c r="D16" s="26">
         <v>295424</v>
       </c>
-      <c r="E16" s="8">
-        <v>0</v>
-      </c>
-      <c r="F16" s="8">
+      <c r="E16" s="26">
+        <v>0</v>
+      </c>
+      <c r="F16" s="26">
         <v>295424</v>
       </c>
-      <c r="G16" s="7">
+      <c r="G16" s="25">
         <v>126</v>
       </c>
-      <c r="H16" s="8">
+      <c r="H16" s="26">
         <v>295424</v>
       </c>
-      <c r="I16" s="8">
+      <c r="I16" s="26">
         <v>265500</v>
       </c>
-      <c r="J16" s="7">
+      <c r="J16" s="25">
         <v>137</v>
       </c>
-      <c r="K16" s="8">
+      <c r="K16" s="26">
         <v>29924</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A17" s="5" t="s">
+    <row r="17" spans="1:11" ht="23" customHeight="1">
+      <c r="A17" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="C17" s="5">
+      <c r="C17" s="22">
         <v>27</v>
       </c>
-      <c r="D17" s="6">
+      <c r="D17" s="23">
         <v>205500</v>
       </c>
-      <c r="E17" s="6">
+      <c r="E17" s="23">
         <v>159500</v>
       </c>
-      <c r="F17" s="6">
+      <c r="F17" s="23">
         <v>46000</v>
       </c>
-      <c r="G17" s="5">
+      <c r="G17" s="22">
         <v>17</v>
       </c>
-      <c r="H17" s="6">
+      <c r="H17" s="23">
         <v>187000</v>
       </c>
-      <c r="I17" s="6">
+      <c r="I17" s="23">
         <v>35000</v>
       </c>
-      <c r="J17" s="5">
+      <c r="J17" s="22">
         <v>20</v>
       </c>
-      <c r="K17" s="6">
+      <c r="K17" s="23">
         <v>11000</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A18" s="9" t="s">
+    <row r="18" spans="1:11" ht="23" customHeight="1">
+      <c r="A18" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="B18" s="9" t="s">
+      <c r="B18" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="C18" s="9">
+      <c r="C18" s="27">
         <v>74</v>
       </c>
-      <c r="D18" s="10">
+      <c r="D18" s="28">
         <v>368543</v>
       </c>
-      <c r="E18" s="10">
-        <v>0</v>
-      </c>
-      <c r="F18" s="10">
+      <c r="E18" s="28">
+        <v>0</v>
+      </c>
+      <c r="F18" s="28">
         <v>368543</v>
       </c>
-      <c r="G18" s="9">
+      <c r="G18" s="27">
         <v>69</v>
       </c>
-      <c r="H18" s="10">
+      <c r="H18" s="28">
         <v>360548</v>
       </c>
-      <c r="I18" s="10">
+      <c r="I18" s="28">
         <v>141100</v>
       </c>
-      <c r="J18" s="9">
+      <c r="J18" s="27">
         <v>73</v>
       </c>
-      <c r="K18" s="10">
+      <c r="K18" s="28">
         <v>227443</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A19" s="7" t="s">
+    <row r="19" spans="1:11" ht="23" customHeight="1">
+      <c r="A19" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B19" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="C19" s="7">
+      <c r="C19" s="25">
         <v>158</v>
       </c>
-      <c r="D19" s="8">
+      <c r="D19" s="26">
         <v>359128</v>
       </c>
-      <c r="E19" s="8">
-        <v>0</v>
-      </c>
-      <c r="F19" s="8">
+      <c r="E19" s="26">
+        <v>0</v>
+      </c>
+      <c r="F19" s="26">
         <v>359128</v>
       </c>
-      <c r="G19" s="7">
+      <c r="G19" s="25">
         <v>155</v>
       </c>
-      <c r="H19" s="8">
+      <c r="H19" s="26">
         <v>355128</v>
       </c>
-      <c r="I19" s="8">
+      <c r="I19" s="26">
         <v>316300</v>
       </c>
-      <c r="J19" s="7">
+      <c r="J19" s="25">
         <v>164</v>
       </c>
-      <c r="K19" s="8">
+      <c r="K19" s="26">
         <v>42828</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A20" s="5" t="s">
+    <row r="20" spans="1:11" ht="23" customHeight="1">
+      <c r="A20" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="C20" s="5">
+      <c r="C20" s="22">
         <v>72</v>
       </c>
-      <c r="D20" s="6">
+      <c r="D20" s="23">
         <v>2813000</v>
       </c>
-      <c r="E20" s="6">
+      <c r="E20" s="23">
         <v>2668000</v>
       </c>
-      <c r="F20" s="6">
+      <c r="F20" s="23">
         <v>145000</v>
       </c>
-      <c r="G20" s="5">
+      <c r="G20" s="22">
         <v>69</v>
       </c>
-      <c r="H20" s="6">
+      <c r="H20" s="23">
         <v>2808000</v>
       </c>
-      <c r="I20" s="6">
+      <c r="I20" s="23">
         <v>158000</v>
       </c>
-      <c r="J20" s="5">
+      <c r="J20" s="22">
         <v>83</v>
       </c>
-      <c r="K20" s="6">
+      <c r="K20" s="23">
         <v>-13000</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A21" s="9" t="s">
+    <row r="21" spans="1:11" ht="23" customHeight="1">
+      <c r="A21" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="B21" s="9" t="s">
+      <c r="B21" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="C21" s="9">
+      <c r="C21" s="27">
         <v>49</v>
       </c>
-      <c r="D21" s="10">
+      <c r="D21" s="28">
         <v>371340</v>
       </c>
-      <c r="E21" s="10">
-        <v>0</v>
-      </c>
-      <c r="F21" s="10">
+      <c r="E21" s="28">
+        <v>0</v>
+      </c>
+      <c r="F21" s="28">
         <v>371340</v>
       </c>
-      <c r="G21" s="9">
+      <c r="G21" s="27">
         <v>26</v>
       </c>
-      <c r="H21" s="10">
+      <c r="H21" s="28">
         <v>322340</v>
       </c>
-      <c r="I21" s="10">
+      <c r="I21" s="28">
         <v>112300</v>
       </c>
-      <c r="J21" s="9">
+      <c r="J21" s="27">
         <v>59</v>
       </c>
-      <c r="K21" s="10">
+      <c r="K21" s="28">
         <v>259040</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A22" s="7" t="s">
+    <row r="22" spans="1:11" ht="23" customHeight="1">
+      <c r="A22" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="B22" s="7" t="s">
+      <c r="B22" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="C22" s="7">
+      <c r="C22" s="25">
         <v>319</v>
       </c>
-      <c r="D22" s="8">
+      <c r="D22" s="26">
         <v>746670</v>
       </c>
-      <c r="E22" s="8">
-        <v>0</v>
-      </c>
-      <c r="F22" s="8">
+      <c r="E22" s="26">
+        <v>0</v>
+      </c>
+      <c r="F22" s="26">
         <v>746670</v>
       </c>
-      <c r="G22" s="7">
+      <c r="G22" s="25">
         <v>295</v>
       </c>
-      <c r="H22" s="8">
+      <c r="H22" s="26">
         <v>704191</v>
       </c>
-      <c r="I22" s="8">
+      <c r="I22" s="26">
         <v>688100</v>
       </c>
-      <c r="J22" s="7">
+      <c r="J22" s="25">
         <v>362</v>
       </c>
-      <c r="K22" s="8">
+      <c r="K22" s="26">
         <v>58570</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A23" s="5" t="s">
+    <row r="23" spans="1:11" ht="23" customHeight="1">
+      <c r="A23" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B23" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="C23" s="5">
+      <c r="C23" s="22">
         <v>39</v>
       </c>
-      <c r="D23" s="6">
+      <c r="D23" s="23">
         <v>1928000</v>
       </c>
-      <c r="E23" s="6">
+      <c r="E23" s="23">
         <v>1862000</v>
       </c>
-      <c r="F23" s="6">
+      <c r="F23" s="23">
         <v>66000</v>
       </c>
-      <c r="G23" s="5">
+      <c r="G23" s="22">
         <v>39</v>
       </c>
-      <c r="H23" s="6">
+      <c r="H23" s="23">
         <v>1928000</v>
       </c>
-      <c r="I23" s="6">
+      <c r="I23" s="23">
         <v>78000</v>
       </c>
-      <c r="J23" s="5">
+      <c r="J23" s="22">
         <v>40</v>
       </c>
-      <c r="K23" s="6">
+      <c r="K23" s="23">
         <v>-12000</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A24" s="9" t="s">
+    <row r="24" spans="1:11" ht="23" customHeight="1">
+      <c r="A24" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="B24" s="9" t="s">
+      <c r="B24" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="C24" s="9">
+      <c r="C24" s="27">
         <v>87</v>
       </c>
-      <c r="D24" s="10">
+      <c r="D24" s="28">
         <v>487568</v>
       </c>
-      <c r="E24" s="10">
-        <v>0</v>
-      </c>
-      <c r="F24" s="10">
+      <c r="E24" s="28">
+        <v>0</v>
+      </c>
+      <c r="F24" s="28">
         <v>487568</v>
       </c>
-      <c r="G24" s="9">
+      <c r="G24" s="27">
         <v>80</v>
       </c>
-      <c r="H24" s="10">
+      <c r="H24" s="28">
         <v>463868</v>
       </c>
-      <c r="I24" s="10">
+      <c r="I24" s="28">
         <v>193200</v>
       </c>
-      <c r="J24" s="9">
+      <c r="J24" s="27">
         <v>99</v>
       </c>
-      <c r="K24" s="10">
+      <c r="K24" s="28">
         <v>294368</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A25" s="9" t="s">
+    <row r="25" spans="1:11" ht="23" customHeight="1">
+      <c r="A25" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="B25" s="9" t="s">
+      <c r="B25" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="C25" s="9">
+      <c r="C25" s="27">
         <v>286</v>
       </c>
-      <c r="D25" s="10">
+      <c r="D25" s="28">
         <v>588803</v>
       </c>
-      <c r="E25" s="10">
-        <v>0</v>
-      </c>
-      <c r="F25" s="10">
+      <c r="E25" s="28">
+        <v>0</v>
+      </c>
+      <c r="F25" s="28">
         <v>588803</v>
       </c>
-      <c r="G25" s="9">
+      <c r="G25" s="27">
         <v>230</v>
       </c>
-      <c r="H25" s="10">
+      <c r="H25" s="28">
         <v>499845</v>
       </c>
-      <c r="I25" s="10">
+      <c r="I25" s="28">
         <v>357300</v>
       </c>
-      <c r="J25" s="9">
+      <c r="J25" s="27">
         <v>189</v>
       </c>
-      <c r="K25" s="10">
+      <c r="K25" s="28">
         <v>231503</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A26" s="5" t="s">
+    <row r="26" spans="1:11" ht="23" customHeight="1">
+      <c r="A26" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="B26" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="C26" s="5">
+      <c r="C26" s="22">
         <v>57</v>
       </c>
-      <c r="D26" s="6">
+      <c r="D26" s="23">
         <v>973300</v>
       </c>
-      <c r="E26" s="6">
+      <c r="E26" s="23">
         <v>856000</v>
       </c>
-      <c r="F26" s="6">
+      <c r="F26" s="23">
         <v>117300</v>
       </c>
-      <c r="G26" s="5">
+      <c r="G26" s="22">
         <v>53</v>
       </c>
-      <c r="H26" s="6">
+      <c r="H26" s="23">
         <v>121800</v>
       </c>
-      <c r="I26" s="6">
+      <c r="I26" s="23">
         <v>123800</v>
       </c>
-      <c r="J26" s="5">
+      <c r="J26" s="22">
         <v>65</v>
       </c>
-      <c r="K26" s="6">
+      <c r="K26" s="23">
         <v>-6500</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A27" s="9" t="s">
+    <row r="27" spans="1:11" ht="23" customHeight="1">
+      <c r="A27" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="B27" s="9" t="s">
+      <c r="B27" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="C27" s="9">
+      <c r="C27" s="27">
         <v>62</v>
       </c>
-      <c r="D27" s="10">
+      <c r="D27" s="28">
         <v>321435</v>
       </c>
-      <c r="E27" s="10">
-        <v>0</v>
-      </c>
-      <c r="F27" s="10">
+      <c r="E27" s="28">
+        <v>0</v>
+      </c>
+      <c r="F27" s="28">
         <v>321435</v>
       </c>
-      <c r="G27" s="9">
+      <c r="G27" s="27">
         <v>51</v>
       </c>
-      <c r="H27" s="10">
+      <c r="H27" s="28">
         <v>212555</v>
       </c>
-      <c r="I27" s="10">
+      <c r="I27" s="28">
         <v>116000</v>
       </c>
-      <c r="J27" s="9">
+      <c r="J27" s="27">
         <v>59</v>
       </c>
-      <c r="K27" s="10">
+      <c r="K27" s="28">
         <v>205435</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A28" s="7" t="s">
+    <row r="28" spans="1:11" ht="23" customHeight="1">
+      <c r="A28" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="B28" s="7" t="s">
+      <c r="B28" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="C28" s="7">
+      <c r="C28" s="25">
         <v>343</v>
       </c>
-      <c r="D28" s="8">
+      <c r="D28" s="26">
         <v>799501</v>
       </c>
-      <c r="E28" s="8">
-        <v>0</v>
-      </c>
-      <c r="F28" s="8">
+      <c r="E28" s="26">
+        <v>0</v>
+      </c>
+      <c r="F28" s="26">
         <v>799501</v>
       </c>
-      <c r="G28" s="7">
+      <c r="G28" s="25">
         <v>337</v>
       </c>
-      <c r="H28" s="8">
+      <c r="H28" s="26">
         <v>783501</v>
       </c>
-      <c r="I28" s="8">
+      <c r="I28" s="26">
         <v>861553</v>
       </c>
-      <c r="J28" s="7">
+      <c r="J28" s="25">
         <v>442</v>
       </c>
-      <c r="K28" s="8">
+      <c r="K28" s="26">
         <v>-62052</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A29" s="7" t="s">
+    <row r="29" spans="1:11" ht="23" customHeight="1">
+      <c r="A29" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="B29" s="7" t="s">
+      <c r="B29" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="C29" s="7">
+      <c r="C29" s="25">
         <v>72</v>
       </c>
-      <c r="D29" s="8">
+      <c r="D29" s="26">
         <v>190200</v>
       </c>
-      <c r="E29" s="8">
+      <c r="E29" s="26">
         <v>23700</v>
       </c>
-      <c r="F29" s="8">
+      <c r="F29" s="26">
         <v>166500</v>
       </c>
-      <c r="G29" s="7">
+      <c r="G29" s="25">
         <v>67</v>
       </c>
-      <c r="H29" s="8">
+      <c r="H29" s="26">
         <v>181200</v>
       </c>
-      <c r="I29" s="8">
+      <c r="I29" s="26">
         <v>189200</v>
       </c>
-      <c r="J29" s="7">
+      <c r="J29" s="25">
         <v>98</v>
       </c>
-      <c r="K29" s="8">
+      <c r="K29" s="26">
         <v>-22700</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A30" s="9" t="s">
+    <row r="30" spans="1:11" ht="23" customHeight="1">
+      <c r="A30" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="B30" s="9" t="s">
+      <c r="B30" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="C30" s="9">
+      <c r="C30" s="27">
         <v>14</v>
       </c>
-      <c r="D30" s="10">
+      <c r="D30" s="28">
         <v>155654</v>
       </c>
-      <c r="E30" s="10">
-        <v>0</v>
-      </c>
-      <c r="F30" s="10">
+      <c r="E30" s="28">
+        <v>0</v>
+      </c>
+      <c r="F30" s="28">
         <v>155654</v>
       </c>
-      <c r="G30" s="9">
+      <c r="G30" s="27">
         <v>11</v>
       </c>
-      <c r="H30" s="10">
+      <c r="H30" s="28">
         <v>149654</v>
       </c>
-      <c r="I30" s="10">
+      <c r="I30" s="28">
         <v>38000</v>
       </c>
-      <c r="J30" s="9">
+      <c r="J30" s="27">
         <v>19</v>
       </c>
-      <c r="K30" s="10">
+      <c r="K30" s="28">
         <v>117654</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K1"/>
+  <autoFilter ref="A1:K1" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <phoneticPr fontId="3"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E21"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -2348,7 +2404,7 @@
     <col min="5" max="5" width="70" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" s="3" customFormat="1">
       <c r="A1" s="4" t="s">
         <v>5</v>
       </c>
@@ -2365,7 +2421,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5">
       <c r="A2" s="7" t="s">
         <v>10</v>
       </c>
@@ -2382,7 +2438,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5">
       <c r="A3" s="7" t="s">
         <v>12</v>
       </c>
@@ -2399,7 +2455,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5">
       <c r="A4" s="5" t="s">
         <v>13</v>
       </c>
@@ -2416,7 +2472,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5">
       <c r="A5" s="7" t="s">
         <v>13</v>
       </c>
@@ -2433,7 +2489,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5">
       <c r="A6" s="5" t="s">
         <v>14</v>
       </c>
@@ -2450,7 +2506,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5">
       <c r="A7" s="7" t="s">
         <v>14</v>
       </c>
@@ -2467,7 +2523,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5">
       <c r="A8" s="5" t="s">
         <v>15</v>
       </c>
@@ -2484,7 +2540,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5">
       <c r="A9" s="7" t="s">
         <v>15</v>
       </c>
@@ -2501,7 +2557,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5">
       <c r="A10" s="5" t="s">
         <v>16</v>
       </c>
@@ -2518,7 +2574,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5">
       <c r="A11" s="7" t="s">
         <v>16</v>
       </c>
@@ -2535,7 +2591,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5">
       <c r="A12" s="5" t="s">
         <v>17</v>
       </c>
@@ -2552,7 +2608,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5">
       <c r="A13" s="7" t="s">
         <v>17</v>
       </c>
@@ -2569,7 +2625,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5">
       <c r="A14" s="7" t="s">
         <v>18</v>
       </c>
@@ -2586,7 +2642,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5">
       <c r="A15" s="5" t="s">
         <v>18</v>
       </c>
@@ -2603,7 +2659,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5">
       <c r="A16" s="5" t="s">
         <v>19</v>
       </c>
@@ -2620,7 +2676,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5">
       <c r="A17" s="5" t="s">
         <v>19</v>
       </c>
@@ -2637,7 +2693,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5">
       <c r="A18" s="7" t="s">
         <v>19</v>
       </c>
@@ -2654,7 +2710,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5">
       <c r="A19" s="5" t="s">
         <v>20</v>
       </c>
@@ -2671,7 +2727,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5">
       <c r="A20" s="7" t="s">
         <v>20</v>
       </c>
@@ -2688,7 +2744,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5">
       <c r="A21" s="5" t="s">
         <v>21</v>
       </c>
@@ -2706,22 +2762,23 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E1"/>
+  <autoFilter ref="A1:E1" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
+  <phoneticPr fontId="3"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="2" width="104" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" s="3" customFormat="1">
       <c r="A1" s="4" t="s">
         <v>41</v>
       </c>
@@ -2729,7 +2786,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2">
       <c r="A2" t="s">
         <v>43</v>
       </c>
@@ -2737,7 +2794,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2">
       <c r="A3" t="s">
         <v>45</v>
       </c>
@@ -2745,7 +2802,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2">
       <c r="A4" t="s">
         <v>26</v>
       </c>
@@ -2753,7 +2810,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2">
       <c r="A5" t="s">
         <v>48</v>
       </c>
@@ -2761,7 +2818,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2">
       <c r="A6" t="s">
         <v>50</v>
       </c>
@@ -2770,7 +2827,8 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: đối soát sao kê ở mức từng giao dịch, ghép theo lần thu
Bảng theo tháng chỉ nói tháng nào lệch bao nhiêu, không chỉ được lệch ở giao
dịch nào. Trang "Từng giao dịch" đặt mỗi dòng sao kê cạnh khoản thu bên phần
mềm, tô màu theo độ chắc của phép ghép.

Đơn vị ghép bên phần mềm là LẦN THU — các đợt cùng hợp đồng, cùng ngày thu —
chứ không phải từng đợt, vì khách hay đóng gộp mấy kỳ một lần: 473 lần thu
gộp, 1.152 đợt, hơn hai triệu. Ghép từng đợt một thì cả nhóm đó không bao giờ
khớp; đổi sang lần thu, số ghép được lên từ 2.984.452 thành 4.294.653 và số
đợt chưa ghép giảm từ 1.270 xuống 556.

Một giao dịch ghép đúng một lần thu, một đợt chỉ nằm trong một cặp — ràng
buộc này có test riêng, vì lần trước thiếu nó nên một khoản 1.100 bị gán cho
cả ba kỳ 10, 11, 12 của cùng hợp đồng.

File xuất tự đánh version v1, v2, v3 nên chạy lại không đè bản cũ.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/sao-ke-co-dinh-theo-thang-va-tai-khoan.xlsx
+++ b/data/sao-ke-co-dinh-theo-thang-va-tai-khoan.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10914"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D03A6C8-BD96-4346-A81F-FF01D7ED9D12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E9594B0-7E98-914A-874C-CF03C1536E52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="41120" windowHeight="24600" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="41120" windowHeight="24600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Theo tháng và tài khoản" sheetId="1" r:id="rId1"/>
@@ -180,7 +180,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -196,20 +196,75 @@
       <charset val="128"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <name val="ＭＳ Ｐゴシック"/>
-      <charset val="128"/>
-    </font>
-    <font>
       <sz val="6"/>
       <name val="ＭＳ Ｐゴシック"/>
       <family val="3"/>
       <charset val="128"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF006100"/>
+      <name val="ＭＳ Ｐゴシック"/>
+      <family val="2"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF9C0006"/>
+      <name val="ＭＳ Ｐゴシック"/>
+      <family val="2"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF9C5700"/>
+      <name val="ＭＳ Ｐゴシック"/>
+      <family val="2"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Consolas"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF9C5700"/>
+      <name val="Consolas"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF9C0006"/>
+      <name val="Consolas"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF006100"/>
+      <name val="Consolas"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Consolas"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Consolas"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -246,8 +301,23 @@
         <fgColor rgb="FFDCE6F1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -255,37 +325,45 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="3" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="3" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="3" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="3" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="3" fontId="2" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -318,9 +396,75 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="11" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="4">
+    <cellStyle name="どちらでもない" xfId="3" builtinId="28"/>
+    <cellStyle name="悪い" xfId="2" builtinId="27"/>
     <cellStyle name="標準" xfId="0" builtinId="0"/>
+    <cellStyle name="良い" xfId="1" builtinId="26"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -658,649 +802,648 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M16"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="13.33203125" defaultRowHeight="26" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="13" width="14" customWidth="1"/>
+    <col min="1" max="16384" width="13.33203125" style="21"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="1" customFormat="1">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="18" t="s">
+    <row r="1" spans="1:13" s="20" customFormat="1" ht="26" customHeight="1">
+      <c r="A1" s="23" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18" t="s">
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18" t="s">
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18" t="s">
+      <c r="I1" s="26"/>
+      <c r="J1" s="26"/>
+      <c r="K1" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
-    </row>
-    <row r="2" spans="1:13" s="3" customFormat="1">
-      <c r="A2" s="4" t="s">
+      <c r="L1" s="27"/>
+      <c r="M1" s="27"/>
+    </row>
+    <row r="2" spans="1:13" s="20" customFormat="1" ht="26" customHeight="1">
+      <c r="A2" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="38" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="39" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="39" t="s">
         <v>8</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="40" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="I2" s="40" t="s">
         <v>7</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="J2" s="40" t="s">
         <v>8</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="K2" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="L2" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="M2" s="4" t="s">
+      <c r="M2" s="23" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="5" t="s">
+    <row r="3" spans="1:13" ht="26" customHeight="1">
+      <c r="A3" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="6">
+      <c r="B3" s="29">
         <v>2500</v>
       </c>
-      <c r="C3" s="6">
-        <v>0</v>
-      </c>
-      <c r="D3" s="6">
+      <c r="C3" s="29">
+        <v>0</v>
+      </c>
+      <c r="D3" s="29">
         <v>2500</v>
       </c>
-      <c r="E3" s="6">
-        <v>0</v>
-      </c>
-      <c r="F3" s="6">
-        <v>0</v>
-      </c>
-      <c r="G3" s="6">
-        <v>0</v>
-      </c>
-      <c r="H3" s="6">
-        <v>0</v>
-      </c>
-      <c r="I3" s="6">
-        <v>0</v>
-      </c>
-      <c r="J3" s="6">
-        <v>0</v>
-      </c>
-      <c r="K3" s="6">
+      <c r="E3" s="29">
+        <v>0</v>
+      </c>
+      <c r="F3" s="29">
+        <v>0</v>
+      </c>
+      <c r="G3" s="29">
+        <v>0</v>
+      </c>
+      <c r="H3" s="29">
+        <v>0</v>
+      </c>
+      <c r="I3" s="29">
+        <v>0</v>
+      </c>
+      <c r="J3" s="29">
+        <v>0</v>
+      </c>
+      <c r="K3" s="29">
         <v>2500</v>
       </c>
-      <c r="L3" s="6">
-        <v>0</v>
-      </c>
-      <c r="M3" s="6">
+      <c r="L3" s="29">
+        <v>0</v>
+      </c>
+      <c r="M3" s="29">
         <v>2500</v>
       </c>
     </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="5" t="s">
+    <row r="4" spans="1:13" ht="26" customHeight="1">
+      <c r="A4" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4" s="29">
         <v>500</v>
       </c>
-      <c r="C4" s="6">
-        <v>0</v>
-      </c>
-      <c r="D4" s="6">
+      <c r="C4" s="29">
+        <v>0</v>
+      </c>
+      <c r="D4" s="29">
         <v>500</v>
       </c>
-      <c r="E4" s="6">
-        <v>0</v>
-      </c>
-      <c r="F4" s="6">
-        <v>0</v>
-      </c>
-      <c r="G4" s="6">
-        <v>0</v>
-      </c>
-      <c r="H4" s="6">
+      <c r="E4" s="29">
+        <v>0</v>
+      </c>
+      <c r="F4" s="29">
+        <v>0</v>
+      </c>
+      <c r="G4" s="29">
+        <v>0</v>
+      </c>
+      <c r="H4" s="29">
         <v>21400</v>
       </c>
-      <c r="I4" s="6">
-        <v>0</v>
-      </c>
-      <c r="J4" s="6">
+      <c r="I4" s="29">
+        <v>0</v>
+      </c>
+      <c r="J4" s="29">
         <v>21400</v>
       </c>
-      <c r="K4" s="6">
+      <c r="K4" s="29">
         <v>21900</v>
       </c>
-      <c r="L4" s="6">
-        <v>0</v>
-      </c>
-      <c r="M4" s="6">
+      <c r="L4" s="29">
+        <v>0</v>
+      </c>
+      <c r="M4" s="29">
         <v>21900</v>
       </c>
     </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="7" t="s">
+    <row r="5" spans="1:13" ht="26" customHeight="1">
+      <c r="A5" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="8">
+      <c r="B5" s="31">
         <v>7700</v>
       </c>
-      <c r="C5" s="8">
-        <v>0</v>
-      </c>
-      <c r="D5" s="8">
+      <c r="C5" s="31">
+        <v>0</v>
+      </c>
+      <c r="D5" s="31">
         <v>7700</v>
       </c>
-      <c r="E5" s="8">
-        <v>0</v>
-      </c>
-      <c r="F5" s="8">
-        <v>0</v>
-      </c>
-      <c r="G5" s="8">
-        <v>0</v>
-      </c>
-      <c r="H5" s="8">
+      <c r="E5" s="31">
+        <v>0</v>
+      </c>
+      <c r="F5" s="31">
+        <v>0</v>
+      </c>
+      <c r="G5" s="31">
+        <v>0</v>
+      </c>
+      <c r="H5" s="31">
         <v>94248</v>
       </c>
-      <c r="I5" s="8">
-        <v>0</v>
-      </c>
-      <c r="J5" s="8">
+      <c r="I5" s="31">
+        <v>0</v>
+      </c>
+      <c r="J5" s="31">
         <v>94248</v>
       </c>
-      <c r="K5" s="8">
+      <c r="K5" s="31">
         <v>101948</v>
       </c>
-      <c r="L5" s="8">
-        <v>0</v>
-      </c>
-      <c r="M5" s="8">
+      <c r="L5" s="31">
+        <v>0</v>
+      </c>
+      <c r="M5" s="31">
         <v>101948</v>
       </c>
     </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="5" t="s">
+    <row r="6" spans="1:13" ht="26" customHeight="1">
+      <c r="A6" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="6">
+      <c r="B6" s="29">
         <v>18850</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="29">
         <v>12000</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="29">
         <v>6850</v>
       </c>
-      <c r="E6" s="6">
-        <v>0</v>
-      </c>
-      <c r="F6" s="6">
-        <v>0</v>
-      </c>
-      <c r="G6" s="6">
-        <v>0</v>
-      </c>
-      <c r="H6" s="6">
+      <c r="E6" s="29">
+        <v>0</v>
+      </c>
+      <c r="F6" s="29">
+        <v>0</v>
+      </c>
+      <c r="G6" s="29">
+        <v>0</v>
+      </c>
+      <c r="H6" s="29">
         <v>143900</v>
       </c>
-      <c r="I6" s="6">
+      <c r="I6" s="29">
         <v>114500</v>
       </c>
-      <c r="J6" s="6">
+      <c r="J6" s="29">
         <v>29400</v>
       </c>
-      <c r="K6" s="6">
+      <c r="K6" s="29">
         <v>162750</v>
       </c>
-      <c r="L6" s="6">
+      <c r="L6" s="29">
         <v>126500</v>
       </c>
-      <c r="M6" s="6">
+      <c r="M6" s="29">
         <v>36250</v>
       </c>
     </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="7" t="s">
+    <row r="7" spans="1:13" ht="26" customHeight="1">
+      <c r="A7" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="8">
+      <c r="B7" s="31">
         <v>18500</v>
       </c>
-      <c r="C7" s="8">
+      <c r="C7" s="31">
         <v>16500</v>
       </c>
-      <c r="D7" s="8">
+      <c r="D7" s="31">
         <v>2000</v>
       </c>
-      <c r="E7" s="8">
-        <v>0</v>
-      </c>
-      <c r="F7" s="8">
-        <v>0</v>
-      </c>
-      <c r="G7" s="8">
-        <v>0</v>
-      </c>
-      <c r="H7" s="8">
+      <c r="E7" s="31">
+        <v>0</v>
+      </c>
+      <c r="F7" s="31">
+        <v>0</v>
+      </c>
+      <c r="G7" s="31">
+        <v>0</v>
+      </c>
+      <c r="H7" s="31">
         <v>158000</v>
       </c>
-      <c r="I7" s="8">
+      <c r="I7" s="31">
         <v>108000</v>
       </c>
-      <c r="J7" s="8">
+      <c r="J7" s="31">
         <v>50000</v>
       </c>
-      <c r="K7" s="8">
+      <c r="K7" s="31">
         <v>176500</v>
       </c>
-      <c r="L7" s="8">
+      <c r="L7" s="31">
         <v>124500</v>
       </c>
-      <c r="M7" s="8">
+      <c r="M7" s="31">
         <v>52000</v>
       </c>
     </row>
-    <row r="8" spans="1:13">
-      <c r="A8" s="9" t="s">
+    <row r="8" spans="1:13" ht="26" customHeight="1">
+      <c r="A8" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="10">
+      <c r="B8" s="33">
         <v>28000</v>
       </c>
-      <c r="C8" s="10">
+      <c r="C8" s="33">
         <v>18000</v>
       </c>
-      <c r="D8" s="10">
+      <c r="D8" s="33">
         <v>10000</v>
       </c>
-      <c r="E8" s="10">
-        <v>0</v>
-      </c>
-      <c r="F8" s="10">
-        <v>0</v>
-      </c>
-      <c r="G8" s="10">
-        <v>0</v>
-      </c>
-      <c r="H8" s="10">
+      <c r="E8" s="33">
+        <v>0</v>
+      </c>
+      <c r="F8" s="33">
+        <v>0</v>
+      </c>
+      <c r="G8" s="33">
+        <v>0</v>
+      </c>
+      <c r="H8" s="33">
         <v>339471</v>
       </c>
-      <c r="I8" s="10">
+      <c r="I8" s="33">
         <v>111600</v>
       </c>
-      <c r="J8" s="10">
+      <c r="J8" s="33">
         <v>227871</v>
       </c>
-      <c r="K8" s="10">
+      <c r="K8" s="33">
         <v>367471</v>
       </c>
-      <c r="L8" s="10">
+      <c r="L8" s="33">
         <v>129600</v>
       </c>
-      <c r="M8" s="10">
+      <c r="M8" s="33">
         <v>237871</v>
       </c>
     </row>
-    <row r="9" spans="1:13">
-      <c r="A9" s="9" t="s">
+    <row r="9" spans="1:13" ht="26" customHeight="1">
+      <c r="A9" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="10">
+      <c r="B9" s="33">
         <v>177469</v>
       </c>
-      <c r="C9" s="10">
+      <c r="C9" s="33">
         <v>189000</v>
       </c>
-      <c r="D9" s="10">
+      <c r="D9" s="33">
         <v>-11531</v>
       </c>
-      <c r="E9" s="10">
-        <v>0</v>
-      </c>
-      <c r="F9" s="10">
+      <c r="E9" s="33">
+        <v>0</v>
+      </c>
+      <c r="F9" s="33">
         <v>2000</v>
       </c>
-      <c r="G9" s="10">
+      <c r="G9" s="33">
         <v>-2000</v>
       </c>
-      <c r="H9" s="10">
+      <c r="H9" s="33">
         <v>540963</v>
       </c>
-      <c r="I9" s="10">
+      <c r="I9" s="33">
         <v>265400</v>
       </c>
-      <c r="J9" s="10">
+      <c r="J9" s="33">
         <v>275563</v>
       </c>
-      <c r="K9" s="10">
+      <c r="K9" s="33">
         <v>718432</v>
       </c>
-      <c r="L9" s="10">
+      <c r="L9" s="33">
         <v>456400</v>
       </c>
-      <c r="M9" s="10">
+      <c r="M9" s="33">
         <v>262032</v>
       </c>
     </row>
-    <row r="10" spans="1:13">
-      <c r="A10" s="9" t="s">
+    <row r="10" spans="1:13" ht="26" customHeight="1">
+      <c r="A10" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="10">
+      <c r="B10" s="33">
         <v>295424</v>
       </c>
-      <c r="C10" s="10">
+      <c r="C10" s="33">
         <v>265500</v>
       </c>
-      <c r="D10" s="10">
+      <c r="D10" s="33">
         <v>29924</v>
       </c>
-      <c r="E10" s="10">
+      <c r="E10" s="33">
         <v>46000</v>
       </c>
-      <c r="F10" s="10">
+      <c r="F10" s="33">
         <v>35000</v>
       </c>
-      <c r="G10" s="10">
+      <c r="G10" s="33">
         <v>11000</v>
       </c>
-      <c r="H10" s="10">
+      <c r="H10" s="33">
         <v>368543</v>
       </c>
-      <c r="I10" s="10">
+      <c r="I10" s="33">
         <v>141100</v>
       </c>
-      <c r="J10" s="10">
+      <c r="J10" s="33">
         <v>227443</v>
       </c>
-      <c r="K10" s="10">
+      <c r="K10" s="33">
         <v>709967</v>
       </c>
-      <c r="L10" s="10">
+      <c r="L10" s="33">
         <v>441600</v>
       </c>
-      <c r="M10" s="10">
+      <c r="M10" s="33">
         <v>268367</v>
       </c>
     </row>
-    <row r="11" spans="1:13">
-      <c r="A11" s="9" t="s">
+    <row r="11" spans="1:13" ht="26" customHeight="1">
+      <c r="A11" s="32" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="10">
+      <c r="B11" s="33">
         <v>359128</v>
       </c>
-      <c r="C11" s="10">
+      <c r="C11" s="33">
         <v>316300</v>
       </c>
-      <c r="D11" s="10">
+      <c r="D11" s="33">
         <v>42828</v>
       </c>
-      <c r="E11" s="10">
+      <c r="E11" s="33">
         <v>145000</v>
       </c>
-      <c r="F11" s="10">
+      <c r="F11" s="33">
         <v>158000</v>
       </c>
-      <c r="G11" s="10">
+      <c r="G11" s="33">
         <v>-13000</v>
       </c>
-      <c r="H11" s="10">
+      <c r="H11" s="33">
         <v>371340</v>
       </c>
-      <c r="I11" s="10">
+      <c r="I11" s="33">
         <v>112300</v>
       </c>
-      <c r="J11" s="10">
+      <c r="J11" s="33">
         <v>259040</v>
       </c>
-      <c r="K11" s="10">
+      <c r="K11" s="33">
         <v>875468</v>
       </c>
-      <c r="L11" s="10">
+      <c r="L11" s="33">
         <v>586600</v>
       </c>
-      <c r="M11" s="10">
+      <c r="M11" s="33">
         <v>288868</v>
       </c>
     </row>
-    <row r="12" spans="1:13">
-      <c r="A12" s="9" t="s">
+    <row r="12" spans="1:13" ht="26" customHeight="1">
+      <c r="A12" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="10">
+      <c r="B12" s="33">
         <v>746670</v>
       </c>
-      <c r="C12" s="10">
+      <c r="C12" s="33">
         <v>688100</v>
       </c>
-      <c r="D12" s="10">
+      <c r="D12" s="33">
         <v>58570</v>
       </c>
-      <c r="E12" s="10">
+      <c r="E12" s="33">
         <v>66000</v>
       </c>
-      <c r="F12" s="10">
+      <c r="F12" s="33">
         <v>78000</v>
       </c>
-      <c r="G12" s="10">
+      <c r="G12" s="33">
         <v>-12000</v>
       </c>
-      <c r="H12" s="10">
+      <c r="H12" s="33">
         <v>487568</v>
       </c>
-      <c r="I12" s="10">
+      <c r="I12" s="33">
         <v>193200</v>
       </c>
-      <c r="J12" s="10">
+      <c r="J12" s="33">
         <v>294368</v>
       </c>
-      <c r="K12" s="10">
+      <c r="K12" s="33">
         <v>1300238</v>
       </c>
-      <c r="L12" s="10">
+      <c r="L12" s="33">
         <v>959300</v>
       </c>
-      <c r="M12" s="10">
+      <c r="M12" s="33">
         <v>340938</v>
       </c>
     </row>
-    <row r="13" spans="1:13">
-      <c r="A13" s="9" t="s">
+    <row r="13" spans="1:13" ht="26" customHeight="1">
+      <c r="A13" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="10">
+      <c r="B13" s="33">
         <v>588803</v>
       </c>
-      <c r="C13" s="10">
+      <c r="C13" s="33">
         <v>357300</v>
       </c>
-      <c r="D13" s="10">
+      <c r="D13" s="33">
         <v>231503</v>
       </c>
-      <c r="E13" s="10">
+      <c r="E13" s="33">
         <v>117300</v>
       </c>
-      <c r="F13" s="10">
+      <c r="F13" s="33">
         <v>123800</v>
       </c>
-      <c r="G13" s="10">
+      <c r="G13" s="33">
         <v>-6500</v>
       </c>
-      <c r="H13" s="10">
+      <c r="H13" s="33">
         <v>321435</v>
       </c>
-      <c r="I13" s="10">
+      <c r="I13" s="33">
         <v>116000</v>
       </c>
-      <c r="J13" s="10">
+      <c r="J13" s="33">
         <v>205435</v>
       </c>
-      <c r="K13" s="10">
+      <c r="K13" s="33">
         <v>1027538</v>
       </c>
-      <c r="L13" s="10">
+      <c r="L13" s="33">
         <v>597100</v>
       </c>
-      <c r="M13" s="10">
+      <c r="M13" s="33">
         <v>430438</v>
       </c>
     </row>
-    <row r="14" spans="1:13">
-      <c r="A14" s="5" t="s">
+    <row r="14" spans="1:13" ht="26" customHeight="1">
+      <c r="A14" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="B14" s="6">
+      <c r="B14" s="29">
         <v>799501</v>
       </c>
-      <c r="C14" s="6">
+      <c r="C14" s="29">
         <v>861553</v>
       </c>
-      <c r="D14" s="6">
+      <c r="D14" s="29">
         <v>-62052</v>
       </c>
-      <c r="E14" s="6">
+      <c r="E14" s="29">
         <v>166500</v>
       </c>
-      <c r="F14" s="6">
+      <c r="F14" s="29">
         <v>189200</v>
       </c>
-      <c r="G14" s="6">
+      <c r="G14" s="29">
         <v>-22700</v>
       </c>
-      <c r="H14" s="6">
+      <c r="H14" s="29">
         <v>155654</v>
       </c>
-      <c r="I14" s="6">
+      <c r="I14" s="29">
         <v>38000</v>
       </c>
-      <c r="J14" s="6">
+      <c r="J14" s="29">
         <v>117654</v>
       </c>
-      <c r="K14" s="6">
+      <c r="K14" s="29">
         <v>1121655</v>
       </c>
-      <c r="L14" s="6">
+      <c r="L14" s="29">
         <v>1088753</v>
       </c>
-      <c r="M14" s="6">
+      <c r="M14" s="29">
         <v>32902</v>
       </c>
     </row>
-    <row r="15" spans="1:13">
-      <c r="A15" s="11" t="s">
+    <row r="15" spans="1:13" ht="26" customHeight="1">
+      <c r="A15" s="34" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="12">
-        <v>0</v>
-      </c>
-      <c r="C15" s="12">
-        <v>0</v>
-      </c>
-      <c r="D15" s="12">
-        <v>0</v>
-      </c>
-      <c r="E15" s="12">
-        <v>0</v>
-      </c>
-      <c r="F15" s="12">
-        <v>0</v>
-      </c>
-      <c r="G15" s="12">
-        <v>0</v>
-      </c>
-      <c r="H15" s="12">
-        <v>0</v>
-      </c>
-      <c r="I15" s="12">
-        <v>0</v>
-      </c>
-      <c r="J15" s="12">
-        <v>0</v>
-      </c>
-      <c r="K15" s="12">
-        <v>0</v>
-      </c>
-      <c r="L15" s="12">
-        <v>0</v>
-      </c>
-      <c r="M15" s="12">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" s="13" customFormat="1">
-      <c r="A16" s="14" t="s">
+      <c r="B15" s="35">
+        <v>0</v>
+      </c>
+      <c r="C15" s="35">
+        <v>0</v>
+      </c>
+      <c r="D15" s="35">
+        <v>0</v>
+      </c>
+      <c r="E15" s="35">
+        <v>0</v>
+      </c>
+      <c r="F15" s="35">
+        <v>0</v>
+      </c>
+      <c r="G15" s="35">
+        <v>0</v>
+      </c>
+      <c r="H15" s="35">
+        <v>0</v>
+      </c>
+      <c r="I15" s="35">
+        <v>0</v>
+      </c>
+      <c r="J15" s="35">
+        <v>0</v>
+      </c>
+      <c r="K15" s="35">
+        <v>0</v>
+      </c>
+      <c r="L15" s="35">
+        <v>0</v>
+      </c>
+      <c r="M15" s="35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" s="22" customFormat="1" ht="26" customHeight="1">
+      <c r="A16" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="B16" s="15">
+      <c r="B16" s="37">
         <v>3043045</v>
       </c>
-      <c r="C16" s="15">
+      <c r="C16" s="37">
         <v>2724253</v>
       </c>
-      <c r="D16" s="15">
+      <c r="D16" s="37">
         <v>318792</v>
       </c>
-      <c r="E16" s="15">
+      <c r="E16" s="37">
         <v>540800</v>
       </c>
-      <c r="F16" s="15">
+      <c r="F16" s="37">
         <v>586000</v>
       </c>
-      <c r="G16" s="15">
+      <c r="G16" s="37">
         <v>-45200</v>
       </c>
-      <c r="H16" s="15">
+      <c r="H16" s="37">
         <v>3002522</v>
       </c>
-      <c r="I16" s="15">
+      <c r="I16" s="37">
         <v>1200100</v>
       </c>
-      <c r="J16" s="15">
+      <c r="J16" s="37">
         <v>1802422</v>
       </c>
-      <c r="K16" s="15">
+      <c r="K16" s="37">
         <v>6586367</v>
       </c>
-      <c r="L16" s="15">
+      <c r="L16" s="37">
         <v>4510353</v>
       </c>
-      <c r="M16" s="15">
+      <c r="M16" s="37">
         <v>2076014</v>
       </c>
     </row>
@@ -1311,7 +1454,7 @@
     <mergeCell ref="H1:J1"/>
     <mergeCell ref="K1:M1"/>
   </mergeCells>
-  <phoneticPr fontId="3"/>
+  <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
@@ -1322,1072 +1465,1072 @@
   <dimension ref="A1:K30"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="23" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="10" style="24" customWidth="1"/>
-    <col min="2" max="2" width="16" style="24" customWidth="1"/>
-    <col min="3" max="3" width="13" style="24" customWidth="1"/>
-    <col min="4" max="5" width="20" style="29" customWidth="1"/>
-    <col min="6" max="6" width="15" style="29" customWidth="1"/>
-    <col min="7" max="7" width="17" style="24" customWidth="1"/>
-    <col min="8" max="8" width="21" style="29" customWidth="1"/>
-    <col min="9" max="9" width="18" style="29" customWidth="1"/>
-    <col min="10" max="10" width="18" style="24" customWidth="1"/>
-    <col min="11" max="11" width="14" style="29" customWidth="1"/>
-    <col min="12" max="16384" width="8.83203125" style="24"/>
+    <col min="1" max="1" width="10" style="14" customWidth="1"/>
+    <col min="2" max="2" width="16" style="14" customWidth="1"/>
+    <col min="3" max="3" width="13" style="14" customWidth="1"/>
+    <col min="4" max="5" width="20" style="19" customWidth="1"/>
+    <col min="6" max="6" width="15" style="19" customWidth="1"/>
+    <col min="7" max="7" width="17" style="14" customWidth="1"/>
+    <col min="8" max="8" width="21" style="19" customWidth="1"/>
+    <col min="9" max="9" width="18" style="19" customWidth="1"/>
+    <col min="10" max="10" width="18" style="14" customWidth="1"/>
+    <col min="11" max="11" width="14" style="19" customWidth="1"/>
+    <col min="12" max="16384" width="8.83203125" style="14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="21" customFormat="1" ht="23" customHeight="1">
-      <c r="A1" s="19" t="s">
+    <row r="1" spans="1:11" s="11" customFormat="1" ht="23" customHeight="1">
+      <c r="A1" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="19" t="s">
+      <c r="B1" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="C1" s="19" t="s">
+      <c r="C1" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="D1" s="20" t="s">
+      <c r="D1" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="E1" s="20" t="s">
+      <c r="E1" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="F1" s="20" t="s">
+      <c r="F1" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="G1" s="19" t="s">
+      <c r="G1" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="H1" s="20" t="s">
+      <c r="H1" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="I1" s="20" t="s">
+      <c r="I1" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="J1" s="19" t="s">
+      <c r="J1" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="K1" s="20" t="s">
+      <c r="K1" s="10" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="23" customHeight="1">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="22">
+      <c r="C2" s="12">
         <v>1</v>
       </c>
-      <c r="D2" s="23">
+      <c r="D2" s="13">
         <v>2500</v>
       </c>
-      <c r="E2" s="23">
-        <v>0</v>
-      </c>
-      <c r="F2" s="23">
+      <c r="E2" s="13">
+        <v>0</v>
+      </c>
+      <c r="F2" s="13">
         <v>2500</v>
       </c>
-      <c r="G2" s="22">
-        <v>0</v>
-      </c>
-      <c r="H2" s="23">
-        <v>0</v>
-      </c>
-      <c r="I2" s="23">
-        <v>0</v>
-      </c>
-      <c r="J2" s="22">
-        <v>0</v>
-      </c>
-      <c r="K2" s="23">
+      <c r="G2" s="12">
+        <v>0</v>
+      </c>
+      <c r="H2" s="13">
+        <v>0</v>
+      </c>
+      <c r="I2" s="13">
+        <v>0</v>
+      </c>
+      <c r="J2" s="12">
+        <v>0</v>
+      </c>
+      <c r="K2" s="13">
         <v>2500</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="23" customHeight="1">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="22">
+      <c r="C3" s="12">
         <v>1</v>
       </c>
-      <c r="D3" s="23">
+      <c r="D3" s="13">
         <v>500</v>
       </c>
-      <c r="E3" s="23">
-        <v>0</v>
-      </c>
-      <c r="F3" s="23">
+      <c r="E3" s="13">
+        <v>0</v>
+      </c>
+      <c r="F3" s="13">
         <v>500</v>
       </c>
-      <c r="G3" s="22">
-        <v>0</v>
-      </c>
-      <c r="H3" s="23">
-        <v>0</v>
-      </c>
-      <c r="I3" s="23">
-        <v>0</v>
-      </c>
-      <c r="J3" s="22">
-        <v>0</v>
-      </c>
-      <c r="K3" s="23">
+      <c r="G3" s="12">
+        <v>0</v>
+      </c>
+      <c r="H3" s="13">
+        <v>0</v>
+      </c>
+      <c r="I3" s="13">
+        <v>0</v>
+      </c>
+      <c r="J3" s="12">
+        <v>0</v>
+      </c>
+      <c r="K3" s="13">
         <v>500</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="23" customHeight="1">
-      <c r="A4" s="25" t="s">
+      <c r="A4" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="25" t="s">
+      <c r="B4" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="25">
+      <c r="C4" s="15">
         <v>6</v>
       </c>
-      <c r="D4" s="26">
+      <c r="D4" s="16">
         <v>21400</v>
       </c>
-      <c r="E4" s="26">
-        <v>0</v>
-      </c>
-      <c r="F4" s="26">
+      <c r="E4" s="16">
+        <v>0</v>
+      </c>
+      <c r="F4" s="16">
         <v>21400</v>
       </c>
-      <c r="G4" s="25">
+      <c r="G4" s="15">
         <v>3</v>
       </c>
-      <c r="H4" s="26">
+      <c r="H4" s="16">
         <v>5500</v>
       </c>
-      <c r="I4" s="26">
-        <v>0</v>
-      </c>
-      <c r="J4" s="25">
-        <v>0</v>
-      </c>
-      <c r="K4" s="26">
+      <c r="I4" s="16">
+        <v>0</v>
+      </c>
+      <c r="J4" s="15">
+        <v>0</v>
+      </c>
+      <c r="K4" s="16">
         <v>21400</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="23" customHeight="1">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="22" t="s">
+      <c r="B5" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="22">
+      <c r="C5" s="12">
         <v>1</v>
       </c>
-      <c r="D5" s="23">
+      <c r="D5" s="13">
         <v>7700</v>
       </c>
-      <c r="E5" s="23">
-        <v>0</v>
-      </c>
-      <c r="F5" s="23">
+      <c r="E5" s="13">
+        <v>0</v>
+      </c>
+      <c r="F5" s="13">
         <v>7700</v>
       </c>
-      <c r="G5" s="22">
-        <v>0</v>
-      </c>
-      <c r="H5" s="23">
-        <v>0</v>
-      </c>
-      <c r="I5" s="23">
-        <v>0</v>
-      </c>
-      <c r="J5" s="22">
-        <v>0</v>
-      </c>
-      <c r="K5" s="23">
+      <c r="G5" s="12">
+        <v>0</v>
+      </c>
+      <c r="H5" s="13">
+        <v>0</v>
+      </c>
+      <c r="I5" s="13">
+        <v>0</v>
+      </c>
+      <c r="J5" s="12">
+        <v>0</v>
+      </c>
+      <c r="K5" s="13">
         <v>7700</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="23" customHeight="1">
-      <c r="A6" s="25" t="s">
+      <c r="A6" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="25" t="s">
+      <c r="B6" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="25">
+      <c r="C6" s="15">
         <v>26</v>
       </c>
-      <c r="D6" s="26">
+      <c r="D6" s="16">
         <v>94248</v>
       </c>
-      <c r="E6" s="26">
-        <v>0</v>
-      </c>
-      <c r="F6" s="26">
+      <c r="E6" s="16">
+        <v>0</v>
+      </c>
+      <c r="F6" s="16">
         <v>94248</v>
       </c>
-      <c r="G6" s="25">
+      <c r="G6" s="15">
         <v>2</v>
       </c>
-      <c r="H6" s="26">
+      <c r="H6" s="16">
         <v>3100</v>
       </c>
-      <c r="I6" s="26">
-        <v>0</v>
-      </c>
-      <c r="J6" s="25">
-        <v>0</v>
-      </c>
-      <c r="K6" s="26">
+      <c r="I6" s="16">
+        <v>0</v>
+      </c>
+      <c r="J6" s="15">
+        <v>0</v>
+      </c>
+      <c r="K6" s="16">
         <v>94248</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="23" customHeight="1">
-      <c r="A7" s="22" t="s">
+      <c r="A7" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="22" t="s">
+      <c r="B7" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C7" s="22">
+      <c r="C7" s="12">
         <v>3</v>
       </c>
-      <c r="D7" s="23">
+      <c r="D7" s="13">
         <v>18850</v>
       </c>
-      <c r="E7" s="23">
-        <v>0</v>
-      </c>
-      <c r="F7" s="23">
+      <c r="E7" s="13">
+        <v>0</v>
+      </c>
+      <c r="F7" s="13">
         <v>18850</v>
       </c>
-      <c r="G7" s="22">
+      <c r="G7" s="12">
         <v>3</v>
       </c>
-      <c r="H7" s="23">
+      <c r="H7" s="13">
         <v>18850</v>
       </c>
-      <c r="I7" s="23">
+      <c r="I7" s="13">
         <v>12000</v>
       </c>
-      <c r="J7" s="22">
+      <c r="J7" s="12">
         <v>6</v>
       </c>
-      <c r="K7" s="23">
+      <c r="K7" s="13">
         <v>6850</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="23" customHeight="1">
-      <c r="A8" s="25" t="s">
+      <c r="A8" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="25" t="s">
+      <c r="B8" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="C8" s="25">
+      <c r="C8" s="15">
         <v>43</v>
       </c>
-      <c r="D8" s="26">
+      <c r="D8" s="16">
         <v>143900</v>
       </c>
-      <c r="E8" s="26">
-        <v>0</v>
-      </c>
-      <c r="F8" s="26">
+      <c r="E8" s="16">
+        <v>0</v>
+      </c>
+      <c r="F8" s="16">
         <v>143900</v>
       </c>
-      <c r="G8" s="25">
+      <c r="G8" s="15">
         <v>42</v>
       </c>
-      <c r="H8" s="26">
+      <c r="H8" s="16">
         <v>141900</v>
       </c>
-      <c r="I8" s="26">
+      <c r="I8" s="16">
         <v>114500</v>
       </c>
-      <c r="J8" s="25">
+      <c r="J8" s="15">
         <v>61</v>
       </c>
-      <c r="K8" s="26">
+      <c r="K8" s="16">
         <v>29400</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="23" customHeight="1">
-      <c r="A9" s="22" t="s">
+      <c r="A9" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="22" t="s">
+      <c r="B9" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C9" s="22">
+      <c r="C9" s="12">
         <v>5</v>
       </c>
-      <c r="D9" s="23">
+      <c r="D9" s="13">
         <v>18500</v>
       </c>
-      <c r="E9" s="23">
-        <v>0</v>
-      </c>
-      <c r="F9" s="23">
+      <c r="E9" s="13">
+        <v>0</v>
+      </c>
+      <c r="F9" s="13">
         <v>18500</v>
       </c>
-      <c r="G9" s="22">
+      <c r="G9" s="12">
         <v>5</v>
       </c>
-      <c r="H9" s="23">
+      <c r="H9" s="13">
         <v>18500</v>
       </c>
-      <c r="I9" s="23">
+      <c r="I9" s="13">
         <v>16500</v>
       </c>
-      <c r="J9" s="22">
+      <c r="J9" s="12">
         <v>9</v>
       </c>
-      <c r="K9" s="23">
+      <c r="K9" s="13">
         <v>2000</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="23" customHeight="1">
-      <c r="A10" s="25" t="s">
+      <c r="A10" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="25" t="s">
+      <c r="B10" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="C10" s="25">
+      <c r="C10" s="15">
         <v>44</v>
       </c>
-      <c r="D10" s="26">
+      <c r="D10" s="16">
         <v>158000</v>
       </c>
-      <c r="E10" s="26">
-        <v>0</v>
-      </c>
-      <c r="F10" s="26">
+      <c r="E10" s="16">
+        <v>0</v>
+      </c>
+      <c r="F10" s="16">
         <v>158000</v>
       </c>
-      <c r="G10" s="25">
+      <c r="G10" s="15">
         <v>43</v>
       </c>
-      <c r="H10" s="26">
+      <c r="H10" s="16">
         <v>146850</v>
       </c>
-      <c r="I10" s="26">
+      <c r="I10" s="16">
         <v>108000</v>
       </c>
-      <c r="J10" s="25">
+      <c r="J10" s="15">
         <v>56</v>
       </c>
-      <c r="K10" s="26">
+      <c r="K10" s="16">
         <v>50000</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="23" customHeight="1">
-      <c r="A11" s="22" t="s">
+      <c r="A11" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="22" t="s">
+      <c r="B11" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C11" s="22">
+      <c r="C11" s="12">
         <v>11</v>
       </c>
-      <c r="D11" s="23">
+      <c r="D11" s="13">
         <v>28000</v>
       </c>
-      <c r="E11" s="23">
-        <v>0</v>
-      </c>
-      <c r="F11" s="23">
+      <c r="E11" s="13">
+        <v>0</v>
+      </c>
+      <c r="F11" s="13">
         <v>28000</v>
       </c>
-      <c r="G11" s="22">
+      <c r="G11" s="12">
         <v>11</v>
       </c>
-      <c r="H11" s="23">
+      <c r="H11" s="13">
         <v>28000</v>
       </c>
-      <c r="I11" s="23">
+      <c r="I11" s="13">
         <v>18000</v>
       </c>
-      <c r="J11" s="22">
+      <c r="J11" s="12">
         <v>9</v>
       </c>
-      <c r="K11" s="23">
+      <c r="K11" s="13">
         <v>10000</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="23" customHeight="1">
-      <c r="A12" s="27" t="s">
+      <c r="A12" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="27" t="s">
+      <c r="B12" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="C12" s="27">
+      <c r="C12" s="17">
         <v>75</v>
       </c>
-      <c r="D12" s="28">
+      <c r="D12" s="18">
         <v>339471</v>
       </c>
-      <c r="E12" s="28">
-        <v>0</v>
-      </c>
-      <c r="F12" s="28">
+      <c r="E12" s="18">
+        <v>0</v>
+      </c>
+      <c r="F12" s="18">
         <v>339471</v>
       </c>
-      <c r="G12" s="27">
+      <c r="G12" s="17">
         <v>71</v>
       </c>
-      <c r="H12" s="28">
+      <c r="H12" s="18">
         <v>307471</v>
       </c>
-      <c r="I12" s="28">
+      <c r="I12" s="18">
         <v>111600</v>
       </c>
-      <c r="J12" s="27">
+      <c r="J12" s="17">
         <v>61</v>
       </c>
-      <c r="K12" s="28">
+      <c r="K12" s="18">
         <v>227871</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="23" customHeight="1">
-      <c r="A13" s="22" t="s">
+      <c r="A13" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="22" t="s">
+      <c r="B13" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C13" s="22">
+      <c r="C13" s="12">
         <v>73</v>
       </c>
-      <c r="D13" s="23">
+      <c r="D13" s="13">
         <v>177469</v>
       </c>
-      <c r="E13" s="23">
-        <v>0</v>
-      </c>
-      <c r="F13" s="23">
+      <c r="E13" s="13">
+        <v>0</v>
+      </c>
+      <c r="F13" s="13">
         <v>177469</v>
       </c>
-      <c r="G13" s="22">
+      <c r="G13" s="12">
         <v>67</v>
       </c>
-      <c r="H13" s="23">
+      <c r="H13" s="13">
         <v>156469</v>
       </c>
-      <c r="I13" s="23">
+      <c r="I13" s="13">
         <v>189000</v>
       </c>
-      <c r="J13" s="22">
+      <c r="J13" s="12">
         <v>101</v>
       </c>
-      <c r="K13" s="23">
+      <c r="K13" s="13">
         <v>-11531</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="23" customHeight="1">
-      <c r="A14" s="22" t="s">
+      <c r="A14" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="22" t="s">
+      <c r="B14" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C14" s="22">
-        <v>0</v>
-      </c>
-      <c r="D14" s="23">
-        <v>0</v>
-      </c>
-      <c r="E14" s="23">
-        <v>0</v>
-      </c>
-      <c r="F14" s="23">
-        <v>0</v>
-      </c>
-      <c r="G14" s="22">
-        <v>0</v>
-      </c>
-      <c r="H14" s="23">
-        <v>0</v>
-      </c>
-      <c r="I14" s="23">
+      <c r="C14" s="12">
+        <v>0</v>
+      </c>
+      <c r="D14" s="13">
+        <v>0</v>
+      </c>
+      <c r="E14" s="13">
+        <v>0</v>
+      </c>
+      <c r="F14" s="13">
+        <v>0</v>
+      </c>
+      <c r="G14" s="12">
+        <v>0</v>
+      </c>
+      <c r="H14" s="13">
+        <v>0</v>
+      </c>
+      <c r="I14" s="13">
         <v>2000</v>
       </c>
-      <c r="J14" s="22">
+      <c r="J14" s="12">
         <v>1</v>
       </c>
-      <c r="K14" s="23">
+      <c r="K14" s="13">
         <v>-2000</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="23" customHeight="1">
-      <c r="A15" s="27" t="s">
+      <c r="A15" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="27" t="s">
+      <c r="B15" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="C15" s="27">
+      <c r="C15" s="17">
         <v>89</v>
       </c>
-      <c r="D15" s="28">
+      <c r="D15" s="18">
         <v>540963</v>
       </c>
-      <c r="E15" s="28">
-        <v>0</v>
-      </c>
-      <c r="F15" s="28">
+      <c r="E15" s="18">
+        <v>0</v>
+      </c>
+      <c r="F15" s="18">
         <v>540963</v>
       </c>
-      <c r="G15" s="27">
+      <c r="G15" s="17">
         <v>87</v>
       </c>
-      <c r="H15" s="28">
+      <c r="H15" s="18">
         <v>532963</v>
       </c>
-      <c r="I15" s="28">
+      <c r="I15" s="18">
         <v>265400</v>
       </c>
-      <c r="J15" s="27">
+      <c r="J15" s="17">
         <v>138</v>
       </c>
-      <c r="K15" s="28">
+      <c r="K15" s="18">
         <v>275563</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="23" customHeight="1">
-      <c r="A16" s="25" t="s">
+      <c r="A16" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="25" t="s">
+      <c r="B16" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="C16" s="25">
+      <c r="C16" s="15">
         <v>126</v>
       </c>
-      <c r="D16" s="26">
+      <c r="D16" s="16">
         <v>295424</v>
       </c>
-      <c r="E16" s="26">
-        <v>0</v>
-      </c>
-      <c r="F16" s="26">
+      <c r="E16" s="16">
+        <v>0</v>
+      </c>
+      <c r="F16" s="16">
         <v>295424</v>
       </c>
-      <c r="G16" s="25">
+      <c r="G16" s="15">
         <v>126</v>
       </c>
-      <c r="H16" s="26">
+      <c r="H16" s="16">
         <v>295424</v>
       </c>
-      <c r="I16" s="26">
+      <c r="I16" s="16">
         <v>265500</v>
       </c>
-      <c r="J16" s="25">
+      <c r="J16" s="15">
         <v>137</v>
       </c>
-      <c r="K16" s="26">
+      <c r="K16" s="16">
         <v>29924</v>
       </c>
     </row>
     <row r="17" spans="1:11" ht="23" customHeight="1">
-      <c r="A17" s="22" t="s">
+      <c r="A17" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="22" t="s">
+      <c r="B17" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C17" s="22">
+      <c r="C17" s="12">
         <v>27</v>
       </c>
-      <c r="D17" s="23">
+      <c r="D17" s="13">
         <v>205500</v>
       </c>
-      <c r="E17" s="23">
+      <c r="E17" s="13">
         <v>159500</v>
       </c>
-      <c r="F17" s="23">
+      <c r="F17" s="13">
         <v>46000</v>
       </c>
-      <c r="G17" s="22">
+      <c r="G17" s="12">
         <v>17</v>
       </c>
-      <c r="H17" s="23">
+      <c r="H17" s="13">
         <v>187000</v>
       </c>
-      <c r="I17" s="23">
+      <c r="I17" s="13">
         <v>35000</v>
       </c>
-      <c r="J17" s="22">
+      <c r="J17" s="12">
         <v>20</v>
       </c>
-      <c r="K17" s="23">
+      <c r="K17" s="13">
         <v>11000</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="23" customHeight="1">
-      <c r="A18" s="27" t="s">
+      <c r="A18" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="B18" s="27" t="s">
+      <c r="B18" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="C18" s="27">
+      <c r="C18" s="17">
         <v>74</v>
       </c>
-      <c r="D18" s="28">
+      <c r="D18" s="18">
         <v>368543</v>
       </c>
-      <c r="E18" s="28">
-        <v>0</v>
-      </c>
-      <c r="F18" s="28">
+      <c r="E18" s="18">
+        <v>0</v>
+      </c>
+      <c r="F18" s="18">
         <v>368543</v>
       </c>
-      <c r="G18" s="27">
+      <c r="G18" s="17">
         <v>69</v>
       </c>
-      <c r="H18" s="28">
+      <c r="H18" s="18">
         <v>360548</v>
       </c>
-      <c r="I18" s="28">
+      <c r="I18" s="18">
         <v>141100</v>
       </c>
-      <c r="J18" s="27">
+      <c r="J18" s="17">
         <v>73</v>
       </c>
-      <c r="K18" s="28">
+      <c r="K18" s="18">
         <v>227443</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="23" customHeight="1">
-      <c r="A19" s="25" t="s">
+      <c r="A19" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="25" t="s">
+      <c r="B19" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="C19" s="25">
+      <c r="C19" s="15">
         <v>158</v>
       </c>
-      <c r="D19" s="26">
+      <c r="D19" s="16">
         <v>359128</v>
       </c>
-      <c r="E19" s="26">
-        <v>0</v>
-      </c>
-      <c r="F19" s="26">
+      <c r="E19" s="16">
+        <v>0</v>
+      </c>
+      <c r="F19" s="16">
         <v>359128</v>
       </c>
-      <c r="G19" s="25">
+      <c r="G19" s="15">
         <v>155</v>
       </c>
-      <c r="H19" s="26">
+      <c r="H19" s="16">
         <v>355128</v>
       </c>
-      <c r="I19" s="26">
+      <c r="I19" s="16">
         <v>316300</v>
       </c>
-      <c r="J19" s="25">
+      <c r="J19" s="15">
         <v>164</v>
       </c>
-      <c r="K19" s="26">
+      <c r="K19" s="16">
         <v>42828</v>
       </c>
     </row>
     <row r="20" spans="1:11" ht="23" customHeight="1">
-      <c r="A20" s="22" t="s">
+      <c r="A20" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="B20" s="22" t="s">
+      <c r="B20" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C20" s="22">
+      <c r="C20" s="12">
         <v>72</v>
       </c>
-      <c r="D20" s="23">
+      <c r="D20" s="13">
         <v>2813000</v>
       </c>
-      <c r="E20" s="23">
+      <c r="E20" s="13">
         <v>2668000</v>
       </c>
-      <c r="F20" s="23">
+      <c r="F20" s="13">
         <v>145000</v>
       </c>
-      <c r="G20" s="22">
+      <c r="G20" s="12">
         <v>69</v>
       </c>
-      <c r="H20" s="23">
+      <c r="H20" s="13">
         <v>2808000</v>
       </c>
-      <c r="I20" s="23">
+      <c r="I20" s="13">
         <v>158000</v>
       </c>
-      <c r="J20" s="22">
+      <c r="J20" s="12">
         <v>83</v>
       </c>
-      <c r="K20" s="23">
+      <c r="K20" s="13">
         <v>-13000</v>
       </c>
     </row>
     <row r="21" spans="1:11" ht="23" customHeight="1">
-      <c r="A21" s="27" t="s">
+      <c r="A21" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="B21" s="27" t="s">
+      <c r="B21" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="C21" s="27">
+      <c r="C21" s="17">
         <v>49</v>
       </c>
-      <c r="D21" s="28">
+      <c r="D21" s="18">
         <v>371340</v>
       </c>
-      <c r="E21" s="28">
-        <v>0</v>
-      </c>
-      <c r="F21" s="28">
+      <c r="E21" s="18">
+        <v>0</v>
+      </c>
+      <c r="F21" s="18">
         <v>371340</v>
       </c>
-      <c r="G21" s="27">
+      <c r="G21" s="17">
         <v>26</v>
       </c>
-      <c r="H21" s="28">
+      <c r="H21" s="18">
         <v>322340</v>
       </c>
-      <c r="I21" s="28">
+      <c r="I21" s="18">
         <v>112300</v>
       </c>
-      <c r="J21" s="27">
+      <c r="J21" s="17">
         <v>59</v>
       </c>
-      <c r="K21" s="28">
+      <c r="K21" s="18">
         <v>259040</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="23" customHeight="1">
-      <c r="A22" s="25" t="s">
+      <c r="A22" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="B22" s="25" t="s">
+      <c r="B22" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="C22" s="25">
+      <c r="C22" s="15">
         <v>319</v>
       </c>
-      <c r="D22" s="26">
+      <c r="D22" s="16">
         <v>746670</v>
       </c>
-      <c r="E22" s="26">
-        <v>0</v>
-      </c>
-      <c r="F22" s="26">
+      <c r="E22" s="16">
+        <v>0</v>
+      </c>
+      <c r="F22" s="16">
         <v>746670</v>
       </c>
-      <c r="G22" s="25">
+      <c r="G22" s="15">
         <v>295</v>
       </c>
-      <c r="H22" s="26">
+      <c r="H22" s="16">
         <v>704191</v>
       </c>
-      <c r="I22" s="26">
+      <c r="I22" s="16">
         <v>688100</v>
       </c>
-      <c r="J22" s="25">
+      <c r="J22" s="15">
         <v>362</v>
       </c>
-      <c r="K22" s="26">
+      <c r="K22" s="16">
         <v>58570</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="23" customHeight="1">
-      <c r="A23" s="22" t="s">
+      <c r="A23" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="B23" s="22" t="s">
+      <c r="B23" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C23" s="22">
+      <c r="C23" s="12">
         <v>39</v>
       </c>
-      <c r="D23" s="23">
+      <c r="D23" s="13">
         <v>1928000</v>
       </c>
-      <c r="E23" s="23">
+      <c r="E23" s="13">
         <v>1862000</v>
       </c>
-      <c r="F23" s="23">
+      <c r="F23" s="13">
         <v>66000</v>
       </c>
-      <c r="G23" s="22">
+      <c r="G23" s="12">
         <v>39</v>
       </c>
-      <c r="H23" s="23">
+      <c r="H23" s="13">
         <v>1928000</v>
       </c>
-      <c r="I23" s="23">
+      <c r="I23" s="13">
         <v>78000</v>
       </c>
-      <c r="J23" s="22">
+      <c r="J23" s="12">
         <v>40</v>
       </c>
-      <c r="K23" s="23">
+      <c r="K23" s="13">
         <v>-12000</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="23" customHeight="1">
-      <c r="A24" s="27" t="s">
+      <c r="A24" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="B24" s="27" t="s">
+      <c r="B24" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="C24" s="27">
+      <c r="C24" s="17">
         <v>87</v>
       </c>
-      <c r="D24" s="28">
+      <c r="D24" s="18">
         <v>487568</v>
       </c>
-      <c r="E24" s="28">
-        <v>0</v>
-      </c>
-      <c r="F24" s="28">
+      <c r="E24" s="18">
+        <v>0</v>
+      </c>
+      <c r="F24" s="18">
         <v>487568</v>
       </c>
-      <c r="G24" s="27">
+      <c r="G24" s="17">
         <v>80</v>
       </c>
-      <c r="H24" s="28">
+      <c r="H24" s="18">
         <v>463868</v>
       </c>
-      <c r="I24" s="28">
+      <c r="I24" s="18">
         <v>193200</v>
       </c>
-      <c r="J24" s="27">
+      <c r="J24" s="17">
         <v>99</v>
       </c>
-      <c r="K24" s="28">
+      <c r="K24" s="18">
         <v>294368</v>
       </c>
     </row>
     <row r="25" spans="1:11" ht="23" customHeight="1">
-      <c r="A25" s="27" t="s">
+      <c r="A25" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="B25" s="27" t="s">
+      <c r="B25" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="C25" s="27">
+      <c r="C25" s="17">
         <v>286</v>
       </c>
-      <c r="D25" s="28">
+      <c r="D25" s="18">
         <v>588803</v>
       </c>
-      <c r="E25" s="28">
-        <v>0</v>
-      </c>
-      <c r="F25" s="28">
+      <c r="E25" s="18">
+        <v>0</v>
+      </c>
+      <c r="F25" s="18">
         <v>588803</v>
       </c>
-      <c r="G25" s="27">
+      <c r="G25" s="17">
         <v>230</v>
       </c>
-      <c r="H25" s="28">
+      <c r="H25" s="18">
         <v>499845</v>
       </c>
-      <c r="I25" s="28">
+      <c r="I25" s="18">
         <v>357300</v>
       </c>
-      <c r="J25" s="27">
+      <c r="J25" s="17">
         <v>189</v>
       </c>
-      <c r="K25" s="28">
+      <c r="K25" s="18">
         <v>231503</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="23" customHeight="1">
-      <c r="A26" s="22" t="s">
+      <c r="A26" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B26" s="22" t="s">
+      <c r="B26" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C26" s="22">
+      <c r="C26" s="12">
         <v>57</v>
       </c>
-      <c r="D26" s="23">
+      <c r="D26" s="13">
         <v>973300</v>
       </c>
-      <c r="E26" s="23">
+      <c r="E26" s="13">
         <v>856000</v>
       </c>
-      <c r="F26" s="23">
+      <c r="F26" s="13">
         <v>117300</v>
       </c>
-      <c r="G26" s="22">
+      <c r="G26" s="12">
         <v>53</v>
       </c>
-      <c r="H26" s="23">
+      <c r="H26" s="13">
         <v>121800</v>
       </c>
-      <c r="I26" s="23">
+      <c r="I26" s="13">
         <v>123800</v>
       </c>
-      <c r="J26" s="22">
+      <c r="J26" s="12">
         <v>65</v>
       </c>
-      <c r="K26" s="23">
+      <c r="K26" s="13">
         <v>-6500</v>
       </c>
     </row>
     <row r="27" spans="1:11" ht="23" customHeight="1">
-      <c r="A27" s="27" t="s">
+      <c r="A27" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="B27" s="27" t="s">
+      <c r="B27" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="C27" s="27">
+      <c r="C27" s="17">
         <v>62</v>
       </c>
-      <c r="D27" s="28">
+      <c r="D27" s="18">
         <v>321435</v>
       </c>
-      <c r="E27" s="28">
-        <v>0</v>
-      </c>
-      <c r="F27" s="28">
+      <c r="E27" s="18">
+        <v>0</v>
+      </c>
+      <c r="F27" s="18">
         <v>321435</v>
       </c>
-      <c r="G27" s="27">
+      <c r="G27" s="17">
         <v>51</v>
       </c>
-      <c r="H27" s="28">
+      <c r="H27" s="18">
         <v>212555</v>
       </c>
-      <c r="I27" s="28">
+      <c r="I27" s="18">
         <v>116000</v>
       </c>
-      <c r="J27" s="27">
+      <c r="J27" s="17">
         <v>59</v>
       </c>
-      <c r="K27" s="28">
+      <c r="K27" s="18">
         <v>205435</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="23" customHeight="1">
-      <c r="A28" s="25" t="s">
+      <c r="A28" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="B28" s="25" t="s">
+      <c r="B28" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="C28" s="25">
+      <c r="C28" s="15">
         <v>343</v>
       </c>
-      <c r="D28" s="26">
+      <c r="D28" s="16">
         <v>799501</v>
       </c>
-      <c r="E28" s="26">
-        <v>0</v>
-      </c>
-      <c r="F28" s="26">
+      <c r="E28" s="16">
+        <v>0</v>
+      </c>
+      <c r="F28" s="16">
         <v>799501</v>
       </c>
-      <c r="G28" s="25">
+      <c r="G28" s="15">
         <v>337</v>
       </c>
-      <c r="H28" s="26">
+      <c r="H28" s="16">
         <v>783501</v>
       </c>
-      <c r="I28" s="26">
+      <c r="I28" s="16">
         <v>861553</v>
       </c>
-      <c r="J28" s="25">
+      <c r="J28" s="15">
         <v>442</v>
       </c>
-      <c r="K28" s="26">
+      <c r="K28" s="16">
         <v>-62052</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="23" customHeight="1">
-      <c r="A29" s="25" t="s">
+      <c r="A29" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="B29" s="25" t="s">
+      <c r="B29" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="C29" s="25">
+      <c r="C29" s="15">
         <v>72</v>
       </c>
-      <c r="D29" s="26">
+      <c r="D29" s="16">
         <v>190200</v>
       </c>
-      <c r="E29" s="26">
+      <c r="E29" s="16">
         <v>23700</v>
       </c>
-      <c r="F29" s="26">
+      <c r="F29" s="16">
         <v>166500</v>
       </c>
-      <c r="G29" s="25">
+      <c r="G29" s="15">
         <v>67</v>
       </c>
-      <c r="H29" s="26">
+      <c r="H29" s="16">
         <v>181200</v>
       </c>
-      <c r="I29" s="26">
+      <c r="I29" s="16">
         <v>189200</v>
       </c>
-      <c r="J29" s="25">
+      <c r="J29" s="15">
         <v>98</v>
       </c>
-      <c r="K29" s="26">
+      <c r="K29" s="16">
         <v>-22700</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="23" customHeight="1">
-      <c r="A30" s="27" t="s">
+      <c r="A30" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="B30" s="27" t="s">
+      <c r="B30" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="C30" s="27">
+      <c r="C30" s="17">
         <v>14</v>
       </c>
-      <c r="D30" s="28">
+      <c r="D30" s="18">
         <v>155654</v>
       </c>
-      <c r="E30" s="28">
-        <v>0</v>
-      </c>
-      <c r="F30" s="28">
+      <c r="E30" s="18">
+        <v>0</v>
+      </c>
+      <c r="F30" s="18">
         <v>155654</v>
       </c>
-      <c r="G30" s="27">
+      <c r="G30" s="17">
         <v>11</v>
       </c>
-      <c r="H30" s="28">
+      <c r="H30" s="18">
         <v>149654</v>
       </c>
-      <c r="I30" s="28">
+      <c r="I30" s="18">
         <v>38000</v>
       </c>
-      <c r="J30" s="27">
+      <c r="J30" s="17">
         <v>19</v>
       </c>
-      <c r="K30" s="28">
+      <c r="K30" s="18">
         <v>117654</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K1" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
-  <phoneticPr fontId="3"/>
+  <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
@@ -2400,370 +2543,370 @@
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="4" max="4" width="15" style="16" customWidth="1"/>
+    <col min="4" max="4" width="15" style="7" customWidth="1"/>
     <col min="5" max="5" width="70" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="3" customFormat="1">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:5" s="1" customFormat="1">
+      <c r="A1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="2" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C2" s="7">
+      <c r="C2" s="5">
         <v>29</v>
       </c>
-      <c r="D2" s="8">
+      <c r="D2" s="6">
         <v>35900</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="5" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C3" s="7">
+      <c r="C3" s="5">
         <v>16</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="6">
         <v>29300</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="5" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="3">
         <v>2</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="4">
         <v>4000</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="3" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C5" s="7">
+      <c r="C5" s="5">
         <v>17</v>
       </c>
-      <c r="D5" s="8">
+      <c r="D5" s="6">
         <v>32200</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="5" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C6" s="5">
+      <c r="C6" s="3">
         <v>3</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="4">
         <v>5000</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="3" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C7" s="7">
+      <c r="C7" s="5">
         <v>26</v>
       </c>
-      <c r="D7" s="8">
+      <c r="D7" s="6">
         <v>48200</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="5" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C8" s="5">
+      <c r="C8" s="3">
         <v>13</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="4">
         <v>26000</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="3" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C9" s="7">
+      <c r="C9" s="5">
         <v>13</v>
       </c>
-      <c r="D9" s="8">
+      <c r="D9" s="6">
         <v>23150</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="5" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C10" s="5">
+      <c r="C10" s="3">
         <v>22</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="4">
         <v>36900</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" s="3" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C11" s="7">
+      <c r="C11" s="5">
         <v>6</v>
       </c>
-      <c r="D11" s="8">
+      <c r="D11" s="6">
         <v>12000</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E11" s="5" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C12" s="5">
+      <c r="C12" s="3">
         <v>49</v>
       </c>
-      <c r="D12" s="6">
+      <c r="D12" s="4">
         <v>87200</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="E12" s="3" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="7" t="s">
+      <c r="A13" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C13" s="7">
+      <c r="C13" s="5">
         <v>4</v>
       </c>
-      <c r="D13" s="8">
+      <c r="D13" s="6">
         <v>8000</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="E13" s="5" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C14" s="7">
+      <c r="C14" s="5">
         <v>3</v>
       </c>
-      <c r="D14" s="8">
+      <c r="D14" s="6">
         <v>6000</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="E14" s="5" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="5" t="s">
+      <c r="A15" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C15" s="5">
+      <c r="C15" s="3">
         <v>58</v>
       </c>
-      <c r="D15" s="6">
+      <c r="D15" s="4">
         <v>105500</v>
       </c>
-      <c r="E15" s="5" t="s">
+      <c r="E15" s="3" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="5" t="s">
+      <c r="A16" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C16" s="5">
+      <c r="C16" s="3">
         <v>110</v>
       </c>
-      <c r="D16" s="6">
+      <c r="D16" s="4">
         <v>195000</v>
       </c>
-      <c r="E16" s="5" t="s">
+      <c r="E16" s="3" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="5" t="s">
+      <c r="A17" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C17" s="5">
+      <c r="C17" s="3">
         <v>2</v>
       </c>
-      <c r="D17" s="6">
+      <c r="D17" s="4">
         <v>4000</v>
       </c>
-      <c r="E17" s="5" t="s">
+      <c r="E17" s="3" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C18" s="7">
+      <c r="C18" s="5">
         <v>3</v>
       </c>
-      <c r="D18" s="8">
+      <c r="D18" s="6">
         <v>6000</v>
       </c>
-      <c r="E18" s="7" t="s">
+      <c r="E18" s="5" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="5" t="s">
+      <c r="A19" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C19" s="5">
+      <c r="C19" s="3">
         <v>49</v>
       </c>
-      <c r="D19" s="6">
+      <c r="D19" s="4">
         <v>85500</v>
       </c>
-      <c r="E19" s="5" t="s">
+      <c r="E19" s="3" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="7" t="s">
+      <c r="A20" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C20" s="7">
+      <c r="C20" s="5">
         <v>1</v>
       </c>
-      <c r="D20" s="8">
+      <c r="D20" s="6">
         <v>2000</v>
       </c>
-      <c r="E20" s="7" t="s">
+      <c r="E20" s="5" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="5" t="s">
+      <c r="A21" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C21" s="5">
+      <c r="C21" s="3">
         <v>2</v>
       </c>
-      <c r="D21" s="6">
+      <c r="D21" s="4">
         <v>4000</v>
       </c>
-      <c r="E21" s="5" t="s">
+      <c r="E21" s="3" t="s">
         <v>38</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:E1" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
-  <phoneticPr fontId="3"/>
+  <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
@@ -2778,11 +2921,11 @@
     <col min="2" max="2" width="104" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="3" customFormat="1">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:2" s="1" customFormat="1">
+      <c r="A1" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="2" t="s">
         <v>42</v>
       </c>
     </row>
@@ -2827,7 +2970,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="3"/>
+  <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>

</xml_diff>